<commit_message>
CRM: update data via web app
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -36001,9 +36001,8 @@
       </c>
     </row>
     <row r="502" hidden="1">
-      <c r="A502">
-        <f>A501+1</f>
-        <v/>
+      <c r="A502" t="n">
+        <v>8597</v>
       </c>
       <c r="B502" t="inlineStr">
         <is>
@@ -36028,10 +36027,6 @@
       </c>
     </row>
     <row r="503" hidden="1">
-      <c r="A503">
-        <f>A502+1</f>
-        <v/>
-      </c>
       <c r="B503" t="inlineStr">
         <is>
           <t>AD Asse</t>
@@ -36055,10 +36050,6 @@
       </c>
     </row>
     <row r="504" hidden="1">
-      <c r="A504">
-        <f>A503+1</f>
-        <v/>
-      </c>
       <c r="B504" t="inlineStr">
         <is>
           <t>AD Ninove</t>
@@ -36082,10 +36073,6 @@
       </c>
     </row>
     <row r="505" hidden="1">
-      <c r="A505">
-        <f>A504+1</f>
-        <v/>
-      </c>
       <c r="B505" t="inlineStr">
         <is>
           <t>AD Brugge Sint Pieters</t>
@@ -36109,10 +36096,6 @@
       </c>
     </row>
     <row r="506" hidden="1">
-      <c r="A506">
-        <f>A505+1</f>
-        <v/>
-      </c>
       <c r="B506" t="inlineStr">
         <is>
           <t>CM Oostende</t>
@@ -36136,10 +36119,6 @@
       </c>
     </row>
     <row r="507" hidden="1">
-      <c r="A507">
-        <f>A506+1</f>
-        <v/>
-      </c>
       <c r="B507" t="inlineStr">
         <is>
           <t>AD Delhaize Borgerhout</t>
@@ -36163,10 +36142,6 @@
       </c>
     </row>
     <row r="508" hidden="1">
-      <c r="A508">
-        <f>A507+1</f>
-        <v/>
-      </c>
       <c r="B508" t="inlineStr">
         <is>
           <t>Proxy Delhaize Staden</t>
@@ -36196,10 +36171,6 @@
       </c>
     </row>
     <row r="509" hidden="1">
-      <c r="A509">
-        <f>A508+1</f>
-        <v/>
-      </c>
       <c r="B509" t="inlineStr">
         <is>
           <t>Proxy Delhaize Langemark</t>
@@ -36229,10 +36200,6 @@
       </c>
     </row>
     <row r="510" hidden="1">
-      <c r="A510">
-        <f>A509+1</f>
-        <v/>
-      </c>
       <c r="B510" t="inlineStr">
         <is>
           <t>CM Elouges</t>
@@ -36262,10 +36229,6 @@
       </c>
     </row>
     <row r="511" hidden="1">
-      <c r="A511">
-        <f>A510+1</f>
-        <v/>
-      </c>
       <c r="B511" t="inlineStr">
         <is>
           <t>CM Alma Herentals</t>
@@ -36295,10 +36258,6 @@
       </c>
     </row>
     <row r="512" hidden="1">
-      <c r="A512">
-        <f>A511+1</f>
-        <v/>
-      </c>
       <c r="B512" t="inlineStr">
         <is>
           <t>Proxy Delhaize Beerzel</t>
@@ -36328,10 +36287,6 @@
       </c>
     </row>
     <row r="513" hidden="1">
-      <c r="A513">
-        <f>A512+1</f>
-        <v/>
-      </c>
       <c r="B513" t="inlineStr">
         <is>
           <t>AD Munsterbilzen</t>
@@ -36361,10 +36316,6 @@
       </c>
     </row>
     <row r="514" hidden="1">
-      <c r="A514">
-        <f>A513+1</f>
-        <v/>
-      </c>
       <c r="B514" t="inlineStr">
         <is>
           <t>AH Schilde</t>
@@ -36394,10 +36345,6 @@
       </c>
     </row>
     <row r="515" hidden="1">
-      <c r="A515">
-        <f>A514+1</f>
-        <v/>
-      </c>
       <c r="B515" t="inlineStr">
         <is>
           <t>AD Barchon</t>
@@ -36427,10 +36374,6 @@
       </c>
     </row>
     <row r="516" hidden="1">
-      <c r="A516">
-        <f>A515+1</f>
-        <v/>
-      </c>
       <c r="B516" t="inlineStr">
         <is>
           <t>AD Hoeilaart</t>
@@ -36460,10 +36403,6 @@
       </c>
     </row>
     <row r="517" hidden="1">
-      <c r="A517">
-        <f>A516+1</f>
-        <v/>
-      </c>
       <c r="B517" t="inlineStr">
         <is>
           <t>AH Merksem</t>
@@ -36493,10 +36432,6 @@
       </c>
     </row>
     <row r="518" hidden="1">
-      <c r="A518">
-        <f>A517+1</f>
-        <v/>
-      </c>
       <c r="B518" t="inlineStr">
         <is>
           <t>CM Oedelem</t>
@@ -36526,10 +36461,6 @@
       </c>
     </row>
     <row r="519" hidden="1">
-      <c r="A519">
-        <f>A518+1</f>
-        <v/>
-      </c>
       <c r="B519" t="inlineStr">
         <is>
           <t>Proxy Delhaize Grootzand</t>
@@ -36559,10 +36490,6 @@
       </c>
     </row>
     <row r="520" hidden="1">
-      <c r="A520">
-        <f>A519+1</f>
-        <v/>
-      </c>
       <c r="B520" t="inlineStr">
         <is>
           <t>Proxy Delhaize Leest</t>
@@ -36592,10 +36519,6 @@
       </c>
     </row>
     <row r="521" hidden="1">
-      <c r="A521">
-        <f>A520+1</f>
-        <v/>
-      </c>
       <c r="B521" t="inlineStr">
         <is>
           <t>AD Zwijnaarde</t>
@@ -36622,10 +36545,6 @@
       </c>
     </row>
     <row r="522" hidden="1">
-      <c r="A522">
-        <f>A521+1</f>
-        <v/>
-      </c>
       <c r="B522" t="inlineStr">
         <is>
           <t>CM St-Gillis-Waas</t>
@@ -36652,10 +36571,6 @@
       </c>
     </row>
     <row r="523" hidden="1">
-      <c r="A523">
-        <f>A522+1</f>
-        <v/>
-      </c>
       <c r="B523" t="inlineStr">
         <is>
           <t>Spar Dadizele</t>
@@ -36685,10 +36600,6 @@
       </c>
     </row>
     <row r="524" hidden="1">
-      <c r="A524">
-        <f>A523+1</f>
-        <v/>
-      </c>
       <c r="B524" t="inlineStr">
         <is>
           <t>Proxy Delhaize Muizen</t>
@@ -36715,10 +36626,6 @@
       </c>
     </row>
     <row r="525" hidden="1">
-      <c r="A525">
-        <f>A524+1</f>
-        <v/>
-      </c>
       <c r="B525" t="inlineStr">
         <is>
           <t>AD Schelle</t>
@@ -36748,10 +36655,6 @@
       </c>
     </row>
     <row r="526" hidden="1">
-      <c r="A526">
-        <f>A525+1</f>
-        <v/>
-      </c>
       <c r="B526" t="inlineStr">
         <is>
           <t>Alvo Kontich</t>
@@ -36781,10 +36684,6 @@
       </c>
     </row>
     <row r="527" hidden="1">
-      <c r="A527">
-        <f>A526+1</f>
-        <v/>
-      </c>
       <c r="B527" t="inlineStr">
         <is>
           <t>Proxy Delhaize Denderhoutem</t>
@@ -36811,10 +36710,6 @@
       </c>
     </row>
     <row r="528" hidden="1">
-      <c r="A528">
-        <f>A527+1</f>
-        <v/>
-      </c>
       <c r="B528" t="inlineStr">
         <is>
           <t>Plus Landgraaf Wetzels</t>
@@ -36844,10 +36739,6 @@
       </c>
     </row>
     <row r="529" hidden="1">
-      <c r="A529">
-        <f>A528+1</f>
-        <v/>
-      </c>
       <c r="B529" t="inlineStr">
         <is>
           <t>AD Roeselare</t>
@@ -36860,10 +36751,6 @@
       </c>
     </row>
     <row r="530" hidden="1">
-      <c r="A530">
-        <f>A529+1</f>
-        <v/>
-      </c>
       <c r="B530" t="inlineStr">
         <is>
           <t>AH Oostende</t>
@@ -36893,10 +36780,6 @@
       </c>
     </row>
     <row r="531" hidden="1">
-      <c r="A531">
-        <f>A530+1</f>
-        <v/>
-      </c>
       <c r="B531" t="inlineStr">
         <is>
           <t>PLUS Simpelveld Schouteten</t>
@@ -36926,10 +36809,6 @@
       </c>
     </row>
     <row r="532" hidden="1">
-      <c r="A532">
-        <f>A531+1</f>
-        <v/>
-      </c>
       <c r="B532" t="inlineStr">
         <is>
           <t>PLUS Simpelveld Schouteten</t>
@@ -36988,10 +36867,6 @@
       </c>
     </row>
     <row r="534" hidden="1">
-      <c r="A534">
-        <f>A533+1</f>
-        <v/>
-      </c>
       <c r="B534" t="inlineStr">
         <is>
           <t>CM Hoboken Zuid</t>
@@ -37021,10 +36896,6 @@
       </c>
     </row>
     <row r="535" hidden="1">
-      <c r="A535">
-        <f>A534+1</f>
-        <v/>
-      </c>
       <c r="B535" t="inlineStr">
         <is>
           <t>CM Hoboken Kiosk</t>
@@ -37054,10 +36925,6 @@
       </c>
     </row>
     <row r="536" hidden="1">
-      <c r="A536">
-        <f>A535+1</f>
-        <v/>
-      </c>
       <c r="B536" t="inlineStr">
         <is>
           <t>CM Meer</t>
@@ -37087,10 +36954,6 @@
       </c>
     </row>
     <row r="537" hidden="1">
-      <c r="A537">
-        <f>A536+1</f>
-        <v/>
-      </c>
       <c r="B537" t="inlineStr">
         <is>
           <t>AH Ninove</t>
@@ -37120,10 +36983,6 @@
       </c>
     </row>
     <row r="538" hidden="1">
-      <c r="A538">
-        <f>A537+1</f>
-        <v/>
-      </c>
       <c r="B538" t="inlineStr">
         <is>
           <t>AH Dendemonde</t>
@@ -37153,10 +37012,6 @@
       </c>
     </row>
     <row r="539" hidden="1">
-      <c r="A539">
-        <f>A538+1</f>
-        <v/>
-      </c>
       <c r="B539" t="inlineStr">
         <is>
           <t>AD Heist-op-den-Berg</t>
@@ -37186,10 +37041,6 @@
       </c>
     </row>
     <row r="540" hidden="1">
-      <c r="A540">
-        <f>A539+1</f>
-        <v/>
-      </c>
       <c r="B540" t="inlineStr">
         <is>
           <t>AH Rumbeke</t>
@@ -37219,10 +37070,6 @@
       </c>
     </row>
     <row r="541" hidden="1">
-      <c r="A541">
-        <f>A540+1</f>
-        <v/>
-      </c>
       <c r="B541" t="inlineStr">
         <is>
           <t>CM Sint-Niklaas</t>
@@ -37252,10 +37099,6 @@
       </c>
     </row>
     <row r="542" hidden="1">
-      <c r="A542">
-        <f>A541+1</f>
-        <v/>
-      </c>
       <c r="B542" t="inlineStr">
         <is>
           <t xml:space="preserve">CM Zeebrugge </t>
@@ -37285,10 +37128,6 @@
       </c>
     </row>
     <row r="543" hidden="1">
-      <c r="A543">
-        <f>A542+1</f>
-        <v/>
-      </c>
       <c r="B543" t="inlineStr">
         <is>
           <t>AD Brecht</t>
@@ -37318,10 +37157,6 @@
       </c>
     </row>
     <row r="544" hidden="1">
-      <c r="A544">
-        <f>A543+1</f>
-        <v/>
-      </c>
       <c r="B544" t="inlineStr">
         <is>
           <t>AD Merksplas</t>
@@ -37351,10 +37186,6 @@
       </c>
     </row>
     <row r="545" hidden="1">
-      <c r="A545">
-        <f>A544+1</f>
-        <v/>
-      </c>
       <c r="B545" t="inlineStr">
         <is>
           <t>AD GrootBijgaarden</t>
@@ -37384,10 +37215,6 @@
       </c>
     </row>
     <row r="546" hidden="1">
-      <c r="A546">
-        <f>A545+1</f>
-        <v/>
-      </c>
       <c r="B546" t="inlineStr">
         <is>
           <t>AD Vichte</t>
@@ -37417,10 +37244,6 @@
       </c>
     </row>
     <row r="547" hidden="1">
-      <c r="A547">
-        <f>A546+1</f>
-        <v/>
-      </c>
       <c r="B547" t="inlineStr">
         <is>
           <t>Proxy Berchem</t>
@@ -37450,10 +37273,6 @@
       </c>
     </row>
     <row r="548" hidden="1">
-      <c r="A548">
-        <f>A547+1</f>
-        <v/>
-      </c>
       <c r="B548" t="inlineStr">
         <is>
           <t>Proxy Berchem</t>
@@ -37483,10 +37302,6 @@
       </c>
     </row>
     <row r="549" hidden="1">
-      <c r="A549">
-        <f>A548+1</f>
-        <v/>
-      </c>
       <c r="B549" t="inlineStr">
         <is>
           <t>JUMBO Eindhoven Boschdijk</t>

</xml_diff>

<commit_message>
Restore original data + re-dedup with correct (invoice#, project) key
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -19994,7 +19994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I560"/>
+  <dimension ref="A1:J666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.5703125" bestFit="1" customWidth="1" style="54" min="1" max="1"/>
@@ -36001,8 +36001,9 @@
       </c>
     </row>
     <row r="502" hidden="1">
-      <c r="A502" t="n">
-        <v>8597</v>
+      <c r="A502">
+        <f>A501+1</f>
+        <v/>
       </c>
       <c r="B502" t="inlineStr">
         <is>
@@ -36027,8 +36028,9 @@
       </c>
     </row>
     <row r="503" hidden="1">
-      <c r="A503" t="n">
-        <v>8598</v>
+      <c r="A503">
+        <f>A502+1</f>
+        <v/>
       </c>
       <c r="B503" t="inlineStr">
         <is>
@@ -36053,8 +36055,9 @@
       </c>
     </row>
     <row r="504" hidden="1">
-      <c r="A504" t="n">
-        <v>8599</v>
+      <c r="A504">
+        <f>A503+1</f>
+        <v/>
       </c>
       <c r="B504" t="inlineStr">
         <is>
@@ -36079,8 +36082,9 @@
       </c>
     </row>
     <row r="505" hidden="1">
-      <c r="A505" t="n">
-        <v>8600</v>
+      <c r="A505">
+        <f>A504+1</f>
+        <v/>
       </c>
       <c r="B505" t="inlineStr">
         <is>
@@ -36105,8 +36109,9 @@
       </c>
     </row>
     <row r="506" hidden="1">
-      <c r="A506" t="n">
-        <v>8601</v>
+      <c r="A506">
+        <f>A505+1</f>
+        <v/>
       </c>
       <c r="B506" t="inlineStr">
         <is>
@@ -36131,8 +36136,9 @@
       </c>
     </row>
     <row r="507" hidden="1">
-      <c r="A507" t="n">
-        <v>8602</v>
+      <c r="A507">
+        <f>A506+1</f>
+        <v/>
       </c>
       <c r="B507" t="inlineStr">
         <is>
@@ -36157,8 +36163,9 @@
       </c>
     </row>
     <row r="508" hidden="1">
-      <c r="A508" t="n">
-        <v>8603</v>
+      <c r="A508">
+        <f>A507+1</f>
+        <v/>
       </c>
       <c r="B508" t="inlineStr">
         <is>
@@ -36189,8 +36196,9 @@
       </c>
     </row>
     <row r="509" hidden="1">
-      <c r="A509" t="n">
-        <v>8604</v>
+      <c r="A509">
+        <f>A508+1</f>
+        <v/>
       </c>
       <c r="B509" t="inlineStr">
         <is>
@@ -36221,8 +36229,9 @@
       </c>
     </row>
     <row r="510" hidden="1">
-      <c r="A510" t="n">
-        <v>8605</v>
+      <c r="A510">
+        <f>A509+1</f>
+        <v/>
       </c>
       <c r="B510" t="inlineStr">
         <is>
@@ -36253,8 +36262,9 @@
       </c>
     </row>
     <row r="511" hidden="1">
-      <c r="A511" t="n">
-        <v>8606</v>
+      <c r="A511">
+        <f>A510+1</f>
+        <v/>
       </c>
       <c r="B511" t="inlineStr">
         <is>
@@ -36285,8 +36295,9 @@
       </c>
     </row>
     <row r="512" hidden="1">
-      <c r="A512" t="n">
-        <v>8607</v>
+      <c r="A512">
+        <f>A511+1</f>
+        <v/>
       </c>
       <c r="B512" t="inlineStr">
         <is>
@@ -36317,8 +36328,9 @@
       </c>
     </row>
     <row r="513" hidden="1">
-      <c r="A513" t="n">
-        <v>8608</v>
+      <c r="A513">
+        <f>A512+1</f>
+        <v/>
       </c>
       <c r="B513" t="inlineStr">
         <is>
@@ -36349,8 +36361,9 @@
       </c>
     </row>
     <row r="514" hidden="1">
-      <c r="A514" t="n">
-        <v>8609</v>
+      <c r="A514">
+        <f>A513+1</f>
+        <v/>
       </c>
       <c r="B514" t="inlineStr">
         <is>
@@ -36381,8 +36394,9 @@
       </c>
     </row>
     <row r="515" hidden="1">
-      <c r="A515" t="n">
-        <v>8610</v>
+      <c r="A515">
+        <f>A514+1</f>
+        <v/>
       </c>
       <c r="B515" t="inlineStr">
         <is>
@@ -36413,8 +36427,9 @@
       </c>
     </row>
     <row r="516" hidden="1">
-      <c r="A516" t="n">
-        <v>8611</v>
+      <c r="A516">
+        <f>A515+1</f>
+        <v/>
       </c>
       <c r="B516" t="inlineStr">
         <is>
@@ -36445,8 +36460,9 @@
       </c>
     </row>
     <row r="517" hidden="1">
-      <c r="A517" t="n">
-        <v>8612</v>
+      <c r="A517">
+        <f>A516+1</f>
+        <v/>
       </c>
       <c r="B517" t="inlineStr">
         <is>
@@ -36477,8 +36493,9 @@
       </c>
     </row>
     <row r="518" hidden="1">
-      <c r="A518" t="n">
-        <v>8613</v>
+      <c r="A518">
+        <f>A517+1</f>
+        <v/>
       </c>
       <c r="B518" t="inlineStr">
         <is>
@@ -36509,8 +36526,9 @@
       </c>
     </row>
     <row r="519" hidden="1">
-      <c r="A519" t="n">
-        <v>8614</v>
+      <c r="A519">
+        <f>A518+1</f>
+        <v/>
       </c>
       <c r="B519" t="inlineStr">
         <is>
@@ -36541,8 +36559,9 @@
       </c>
     </row>
     <row r="520" hidden="1">
-      <c r="A520" t="n">
-        <v>8615</v>
+      <c r="A520">
+        <f>A519+1</f>
+        <v/>
       </c>
       <c r="B520" t="inlineStr">
         <is>
@@ -36573,8 +36592,9 @@
       </c>
     </row>
     <row r="521" hidden="1">
-      <c r="A521" t="n">
-        <v>8616</v>
+      <c r="A521">
+        <f>A520+1</f>
+        <v/>
       </c>
       <c r="B521" t="inlineStr">
         <is>
@@ -36602,8 +36622,9 @@
       </c>
     </row>
     <row r="522" hidden="1">
-      <c r="A522" t="n">
-        <v>8617</v>
+      <c r="A522">
+        <f>A521+1</f>
+        <v/>
       </c>
       <c r="B522" t="inlineStr">
         <is>
@@ -36631,8 +36652,9 @@
       </c>
     </row>
     <row r="523" hidden="1">
-      <c r="A523" t="n">
-        <v>8618</v>
+      <c r="A523">
+        <f>A522+1</f>
+        <v/>
       </c>
       <c r="B523" t="inlineStr">
         <is>
@@ -36663,8 +36685,9 @@
       </c>
     </row>
     <row r="524" hidden="1">
-      <c r="A524" t="n">
-        <v>8619</v>
+      <c r="A524">
+        <f>A523+1</f>
+        <v/>
       </c>
       <c r="B524" t="inlineStr">
         <is>
@@ -36692,8 +36715,9 @@
       </c>
     </row>
     <row r="525" hidden="1">
-      <c r="A525" t="n">
-        <v>8620</v>
+      <c r="A525">
+        <f>A524+1</f>
+        <v/>
       </c>
       <c r="B525" t="inlineStr">
         <is>
@@ -36724,8 +36748,9 @@
       </c>
     </row>
     <row r="526" hidden="1">
-      <c r="A526" t="n">
-        <v>8621</v>
+      <c r="A526">
+        <f>A525+1</f>
+        <v/>
       </c>
       <c r="B526" t="inlineStr">
         <is>
@@ -36756,8 +36781,9 @@
       </c>
     </row>
     <row r="527" hidden="1">
-      <c r="A527" t="n">
-        <v>8622</v>
+      <c r="A527">
+        <f>A526+1</f>
+        <v/>
       </c>
       <c r="B527" t="inlineStr">
         <is>
@@ -36785,8 +36811,9 @@
       </c>
     </row>
     <row r="528" hidden="1">
-      <c r="A528" t="n">
-        <v>8623</v>
+      <c r="A528">
+        <f>A527+1</f>
+        <v/>
       </c>
       <c r="B528" t="inlineStr">
         <is>
@@ -36817,8 +36844,9 @@
       </c>
     </row>
     <row r="529" hidden="1">
-      <c r="A529" t="n">
-        <v>8624</v>
+      <c r="A529">
+        <f>A528+1</f>
+        <v/>
       </c>
       <c r="B529" t="inlineStr">
         <is>
@@ -36832,8 +36860,9 @@
       </c>
     </row>
     <row r="530" hidden="1">
-      <c r="A530" t="n">
-        <v>8625</v>
+      <c r="A530">
+        <f>A529+1</f>
+        <v/>
       </c>
       <c r="B530" t="inlineStr">
         <is>
@@ -36864,8 +36893,9 @@
       </c>
     </row>
     <row r="531" hidden="1">
-      <c r="A531" t="n">
-        <v>8626</v>
+      <c r="A531">
+        <f>A530+1</f>
+        <v/>
       </c>
       <c r="B531" t="inlineStr">
         <is>
@@ -36896,8 +36926,9 @@
       </c>
     </row>
     <row r="532" hidden="1">
-      <c r="A532" t="n">
-        <v>8627</v>
+      <c r="A532">
+        <f>A531+1</f>
+        <v/>
       </c>
       <c r="B532" t="inlineStr">
         <is>
@@ -36957,8 +36988,9 @@
       </c>
     </row>
     <row r="534" hidden="1">
-      <c r="A534" t="n">
-        <v>8629</v>
+      <c r="A534">
+        <f>A533+1</f>
+        <v/>
       </c>
       <c r="B534" t="inlineStr">
         <is>
@@ -36989,8 +37021,9 @@
       </c>
     </row>
     <row r="535" hidden="1">
-      <c r="A535" t="n">
-        <v>8630</v>
+      <c r="A535">
+        <f>A534+1</f>
+        <v/>
       </c>
       <c r="B535" t="inlineStr">
         <is>
@@ -37021,8 +37054,9 @@
       </c>
     </row>
     <row r="536" hidden="1">
-      <c r="A536" t="n">
-        <v>8631</v>
+      <c r="A536">
+        <f>A535+1</f>
+        <v/>
       </c>
       <c r="B536" t="inlineStr">
         <is>
@@ -37053,8 +37087,9 @@
       </c>
     </row>
     <row r="537" hidden="1">
-      <c r="A537" t="n">
-        <v>8632</v>
+      <c r="A537">
+        <f>A536+1</f>
+        <v/>
       </c>
       <c r="B537" t="inlineStr">
         <is>
@@ -37085,8 +37120,9 @@
       </c>
     </row>
     <row r="538" hidden="1">
-      <c r="A538" t="n">
-        <v>8633</v>
+      <c r="A538">
+        <f>A537+1</f>
+        <v/>
       </c>
       <c r="B538" t="inlineStr">
         <is>
@@ -37117,8 +37153,9 @@
       </c>
     </row>
     <row r="539" hidden="1">
-      <c r="A539" t="n">
-        <v>8634</v>
+      <c r="A539">
+        <f>A538+1</f>
+        <v/>
       </c>
       <c r="B539" t="inlineStr">
         <is>
@@ -37149,8 +37186,9 @@
       </c>
     </row>
     <row r="540" hidden="1">
-      <c r="A540" t="n">
-        <v>8635</v>
+      <c r="A540">
+        <f>A539+1</f>
+        <v/>
       </c>
       <c r="B540" t="inlineStr">
         <is>
@@ -37181,8 +37219,9 @@
       </c>
     </row>
     <row r="541" hidden="1">
-      <c r="A541" t="n">
-        <v>8636</v>
+      <c r="A541">
+        <f>A540+1</f>
+        <v/>
       </c>
       <c r="B541" t="inlineStr">
         <is>
@@ -37213,8 +37252,9 @@
       </c>
     </row>
     <row r="542" hidden="1">
-      <c r="A542" t="n">
-        <v>8637</v>
+      <c r="A542">
+        <f>A541+1</f>
+        <v/>
       </c>
       <c r="B542" t="inlineStr">
         <is>
@@ -37245,8 +37285,9 @@
       </c>
     </row>
     <row r="543" hidden="1">
-      <c r="A543" t="n">
-        <v>8638</v>
+      <c r="A543">
+        <f>A542+1</f>
+        <v/>
       </c>
       <c r="B543" t="inlineStr">
         <is>
@@ -37277,8 +37318,9 @@
       </c>
     </row>
     <row r="544" hidden="1">
-      <c r="A544" t="n">
-        <v>8639</v>
+      <c r="A544">
+        <f>A543+1</f>
+        <v/>
       </c>
       <c r="B544" t="inlineStr">
         <is>
@@ -37309,8 +37351,9 @@
       </c>
     </row>
     <row r="545" hidden="1">
-      <c r="A545" t="n">
-        <v>8640</v>
+      <c r="A545">
+        <f>A544+1</f>
+        <v/>
       </c>
       <c r="B545" t="inlineStr">
         <is>
@@ -37341,8 +37384,9 @@
       </c>
     </row>
     <row r="546" hidden="1">
-      <c r="A546" t="n">
-        <v>8641</v>
+      <c r="A546">
+        <f>A545+1</f>
+        <v/>
       </c>
       <c r="B546" t="inlineStr">
         <is>
@@ -37373,8 +37417,9 @@
       </c>
     </row>
     <row r="547" hidden="1">
-      <c r="A547" t="n">
-        <v>8642</v>
+      <c r="A547">
+        <f>A546+1</f>
+        <v/>
       </c>
       <c r="B547" t="inlineStr">
         <is>
@@ -37405,8 +37450,9 @@
       </c>
     </row>
     <row r="548" hidden="1">
-      <c r="A548" t="n">
-        <v>8643</v>
+      <c r="A548">
+        <f>A547+1</f>
+        <v/>
       </c>
       <c r="B548" t="inlineStr">
         <is>
@@ -37437,8 +37483,9 @@
       </c>
     </row>
     <row r="549" hidden="1">
-      <c r="A549" t="n">
-        <v>8644</v>
+      <c r="A549">
+        <f>A548+1</f>
+        <v/>
       </c>
       <c r="B549" t="inlineStr">
         <is>
@@ -37470,147 +37517,151 @@
     </row>
     <row r="550" hidden="1">
       <c r="A550" t="n">
-        <v>8664</v>
+        <v>8670</v>
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>AD Aartselar</t>
+          <t>AD Heverlee</t>
         </is>
       </c>
       <c r="C550" t="inlineStr">
         <is>
-          <t>Y6</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D550" t="n">
-        <v>684</v>
+        <v>7780</v>
       </c>
       <c r="E550" t="n">
-        <v>3</v>
-      </c>
-      <c r="F550" s="201" t="n">
-        <v>45874</v>
+        <v>10</v>
       </c>
       <c r="G550" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H550" t="n">
         <v>2025</v>
       </c>
       <c r="I550" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="551" hidden="1">
       <c r="A551" t="n">
-        <v>8687</v>
+        <v>8670</v>
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>Spar Denderleew (vim3)</t>
+          <t>AD Lovenjoel</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D551" t="n">
-        <v>912</v>
+        <v>7780</v>
       </c>
       <c r="E551" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G551" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="H551" t="n">
+        <v>2025</v>
+      </c>
       <c r="I551" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="552" hidden="1">
       <c r="A552" t="n">
-        <v>8665</v>
+        <v>8670</v>
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>AD Zottegem</t>
+          <t>AD Searena</t>
         </is>
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>Y9</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D552" t="n">
-        <v>1368</v>
+        <v>7780</v>
       </c>
       <c r="E552" t="n">
-        <v>6</v>
-      </c>
-      <c r="F552" s="201" t="n">
-        <v>46044</v>
+        <v>10</v>
       </c>
       <c r="G552" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H552" t="n">
         <v>2025</v>
       </c>
       <c r="I552" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="553" hidden="1">
       <c r="A553" t="n">
-        <v>8666</v>
+        <v>8670</v>
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>AD Zwevegem</t>
+          <t>AD Delhaize Kessel-Lo</t>
         </is>
       </c>
       <c r="C553" t="inlineStr">
         <is>
-          <t>Y2</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D553" t="n">
-        <v>5016</v>
+        <v>7780</v>
       </c>
       <c r="E553" t="n">
-        <v>22</v>
-      </c>
-      <c r="F553" s="201" t="n">
-        <v>46048</v>
+        <v>10</v>
       </c>
       <c r="G553" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H553" t="n">
         <v>2025</v>
       </c>
       <c r="I553" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="554" hidden="1">
       <c r="A554" t="n">
-        <v>8667</v>
+        <v>8670</v>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>AD Delhaize Dessel</t>
+        </is>
       </c>
       <c r="C554" t="inlineStr">
         <is>
-          <t>Y4</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D554" t="n">
-        <v>684</v>
+        <v>7780</v>
       </c>
       <c r="E554" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G554" t="inlineStr">
         <is>
@@ -37621,33 +37672,60 @@
         <v>2025</v>
       </c>
       <c r="I554" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="555" hidden="1">
+      <c r="A555" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>AD Delhaize Tielt-Winge</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D555" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E555" t="n">
+        <v>10</v>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H555" t="n">
+        <v>2025</v>
+      </c>
       <c r="I555" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="556" hidden="1">
       <c r="A556" t="n">
-        <v>8668</v>
+        <v>8670</v>
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>AD Wondelgem</t>
+          <t>Proxy Delhaize Durme</t>
         </is>
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>Y5</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D556" t="n">
-        <v>912</v>
+        <v>7780</v>
       </c>
       <c r="E556" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G556" t="inlineStr">
         <is>
@@ -37658,28 +37736,28 @@
         <v>2025</v>
       </c>
       <c r="I556" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="557" hidden="1">
       <c r="A557" t="n">
-        <v>8669</v>
+        <v>8670</v>
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Rewe Schorn - Bergheim</t>
+          <t>AD Delhaize Wezemaal</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>Paid Trial-0.5Y</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D557" t="n">
-        <v>389</v>
+        <v>7780</v>
       </c>
       <c r="E557" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G557" t="inlineStr">
         <is>
@@ -37689,26 +37767,29 @@
       <c r="H557" t="n">
         <v>2025</v>
       </c>
+      <c r="I557" t="n">
+        <v>778</v>
+      </c>
     </row>
     <row r="558" hidden="1">
       <c r="A558" t="n">
-        <v>8671</v>
+        <v>8670</v>
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>CM Meer</t>
+          <t xml:space="preserve"> Proxy Delhaize Veltem</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
         <is>
-          <t>M-7Y</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D558" t="n">
-        <v>684</v>
+        <v>7780</v>
       </c>
       <c r="E558" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G558" t="inlineStr">
         <is>
@@ -37716,28 +37797,31 @@
         </is>
       </c>
       <c r="H558" t="n">
-        <v>2026</v>
+        <v>2025</v>
+      </c>
+      <c r="I558" t="n">
+        <v>778</v>
       </c>
     </row>
     <row r="559" hidden="1">
       <c r="A559" t="n">
-        <v>8672</v>
+        <v>8670</v>
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>CM Hoboken Zuid</t>
+          <t>AD Delhaize Kluisbergen</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
         <is>
-          <t>M-2Y</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D559" t="n">
-        <v>684</v>
+        <v>7780</v>
       </c>
       <c r="E559" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G559" t="inlineStr">
         <is>
@@ -37745,112 +37829,3471 @@
         </is>
       </c>
       <c r="H559" t="n">
-        <v>2026</v>
+        <v>2025</v>
+      </c>
+      <c r="I559" t="n">
+        <v>778</v>
       </c>
     </row>
     <row r="560" hidden="1">
       <c r="A560" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>AD Delhaize Itegem</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D560" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E560" t="n">
+        <v>10</v>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H560" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I560" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="561" hidden="1">
+      <c r="A561" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>AD Delhaize Pallieter</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D561" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E561" t="n">
+        <v>10</v>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H561" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I561" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="562" hidden="1">
+      <c r="A562" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>AD Delhaize Sint Katelijne Waver</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D562" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E562" t="n">
+        <v>10</v>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H562" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I562" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="563" hidden="1">
+      <c r="A563" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> AD Delhaize Bloemmolens</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D563" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E563" t="n">
+        <v>10</v>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H563" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I563" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="564" hidden="1">
+      <c r="A564" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> AD Delhaize Herselt</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D564" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E564" t="n">
+        <v>10</v>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H564" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I564" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="565" hidden="1">
+      <c r="A565" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>AD Delhaize Hazegras</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D565" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E565" t="n">
+        <v>10</v>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H565" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I565" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="566" hidden="1">
+      <c r="A566" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Delhaize Belval LUXemburg</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D566" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E566" t="n">
+        <v>10</v>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H566" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I566" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="567" hidden="1">
+      <c r="A567" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>AD Aartselar</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D567" t="n">
+        <v>684</v>
+      </c>
+      <c r="E567" t="n">
+        <v>3</v>
+      </c>
+      <c r="F567" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H567" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I567" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="568" hidden="1">
+      <c r="A568" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>AD Nederename</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D568" t="n">
+        <v>684</v>
+      </c>
+      <c r="E568" t="n">
+        <v>3</v>
+      </c>
+      <c r="F568" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H568" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I568" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="569" hidden="1">
+      <c r="A569" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Sint Jan in Eremo</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D569" t="n">
+        <v>684</v>
+      </c>
+      <c r="E569" t="n">
+        <v>3</v>
+      </c>
+      <c r="F569" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H569" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I569" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="570" hidden="1">
+      <c r="A570" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>CM Bascule</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D570" t="n">
+        <v>684</v>
+      </c>
+      <c r="E570" t="n">
+        <v>3</v>
+      </c>
+      <c r="F570" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H570" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I570" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="571" hidden="1">
+      <c r="A571" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>AD Wetteren</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D571" t="n">
+        <v>684</v>
+      </c>
+      <c r="E571" t="n">
+        <v>3</v>
+      </c>
+      <c r="F571" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H571" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I571" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="572" hidden="1">
+      <c r="A572" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>AD Reet</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D572" t="n">
+        <v>684</v>
+      </c>
+      <c r="E572" t="n">
+        <v>3</v>
+      </c>
+      <c r="F572" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H572" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I572" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="573" hidden="1">
+      <c r="A573" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>AD Aalter</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D573" t="n">
+        <v>684</v>
+      </c>
+      <c r="E573" t="n">
+        <v>3</v>
+      </c>
+      <c r="F573" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H573" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I573" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="574" hidden="1">
+      <c r="A574" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>AD Sint-Kruis Brugge</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D574" t="n">
+        <v>684</v>
+      </c>
+      <c r="E574" t="n">
+        <v>3</v>
+      </c>
+      <c r="F574" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H574" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I574" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="575" hidden="1">
+      <c r="A575" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>CM Wilrijk Valaar</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D575" t="n">
+        <v>684</v>
+      </c>
+      <c r="E575" t="n">
+        <v>3</v>
+      </c>
+      <c r="F575" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H575" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I575" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="576" hidden="1">
+      <c r="A576" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>AD Gent Ster</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D576" t="n">
+        <v>684</v>
+      </c>
+      <c r="E576" t="n">
+        <v>3</v>
+      </c>
+      <c r="F576" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H576" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I576" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="577" hidden="1">
+      <c r="A577" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>CM Waregram</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D577" t="n">
+        <v>684</v>
+      </c>
+      <c r="E577" t="n">
+        <v>3</v>
+      </c>
+      <c r="F577" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H577" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I577" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="578" hidden="1">
+      <c r="A578" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Sint-Amandsberg</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D578" t="n">
+        <v>684</v>
+      </c>
+      <c r="E578" t="n">
+        <v>3</v>
+      </c>
+      <c r="F578" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H578" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I578" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="579" hidden="1">
+      <c r="A579" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>CM Essen</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D579" t="n">
+        <v>684</v>
+      </c>
+      <c r="E579" t="n">
+        <v>3</v>
+      </c>
+      <c r="F579" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H579" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I579" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="580" hidden="1">
+      <c r="A580" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>AD Ledeberg</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D580" t="n">
+        <v>684</v>
+      </c>
+      <c r="E580" t="n">
+        <v>3</v>
+      </c>
+      <c r="F580" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H580" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I580" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="581" hidden="1">
+      <c r="A581" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>AD Lede</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D581" t="n">
+        <v>684</v>
+      </c>
+      <c r="E581" t="n">
+        <v>3</v>
+      </c>
+      <c r="F581" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H581" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I581" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="582" hidden="1">
+      <c r="A582" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Sint-Lievens-Houtem</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D582" t="n">
+        <v>684</v>
+      </c>
+      <c r="E582" t="n">
+        <v>3</v>
+      </c>
+      <c r="F582" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H582" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I582" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="583" hidden="1">
+      <c r="A583" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>CM Kapelle-op-den-bos</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D583" t="n">
+        <v>684</v>
+      </c>
+      <c r="E583" t="n">
+        <v>3</v>
+      </c>
+      <c r="F583" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H583" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I583" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="584" hidden="1">
+      <c r="A584" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>AD Deurne</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D584" t="n">
+        <v>684</v>
+      </c>
+      <c r="E584" t="n">
+        <v>3</v>
+      </c>
+      <c r="F584" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H584" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I584" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="585" hidden="1">
+      <c r="A585" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>AD Soumagne</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D585" t="n">
+        <v>684</v>
+      </c>
+      <c r="E585" t="n">
+        <v>3</v>
+      </c>
+      <c r="F585" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H585" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I585" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="586" hidden="1">
+      <c r="A586" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>AD Colfontaine</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D586" t="n">
+        <v>684</v>
+      </c>
+      <c r="E586" t="n">
+        <v>3</v>
+      </c>
+      <c r="F586" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H586" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I586" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="587" hidden="1">
+      <c r="A587" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>AD Galmaarden</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D587" t="n">
+        <v>684</v>
+      </c>
+      <c r="E587" t="n">
+        <v>3</v>
+      </c>
+      <c r="F587" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H587" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I587" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="588" hidden="1">
+      <c r="A588" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>CM Kortenberg</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D588" t="n">
+        <v>684</v>
+      </c>
+      <c r="E588" t="n">
+        <v>3</v>
+      </c>
+      <c r="F588" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H588" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I588" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="589" hidden="1">
+      <c r="A589" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Westkerke</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D589" t="n">
+        <v>684</v>
+      </c>
+      <c r="E589" t="n">
+        <v>3</v>
+      </c>
+      <c r="F589" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H589" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I589" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="590" hidden="1">
+      <c r="A590" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Westerlo</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D590" t="n">
+        <v>684</v>
+      </c>
+      <c r="E590" t="n">
+        <v>3</v>
+      </c>
+      <c r="F590" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H590" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I590" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="591" hidden="1">
+      <c r="A591" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>CM Moorslede</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D591" t="n">
+        <v>684</v>
+      </c>
+      <c r="E591" t="n">
+        <v>3</v>
+      </c>
+      <c r="F591" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H591" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I591" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="592" hidden="1">
+      <c r="A592" t="n">
+        <v>8687</v>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Spar Denderleew (vim3)</t>
+        </is>
+      </c>
+      <c r="D592" t="n">
+        <v>912</v>
+      </c>
+      <c r="E592" t="n">
+        <v>4</v>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I592" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="593" hidden="1">
+      <c r="A593" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>AD Kalmthout</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D593" t="n">
+        <v>684</v>
+      </c>
+      <c r="E593" t="n">
+        <v>3</v>
+      </c>
+      <c r="F593" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H593" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I593" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="594" hidden="1">
+      <c r="A594" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>AD Grimbergen</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D594" t="n">
+        <v>684</v>
+      </c>
+      <c r="E594" t="n">
+        <v>3</v>
+      </c>
+      <c r="F594" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H594" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I594" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="595" hidden="1">
+      <c r="A595" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Veerle</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D595" t="n">
+        <v>684</v>
+      </c>
+      <c r="E595" t="n">
+        <v>3</v>
+      </c>
+      <c r="F595" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H595" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I595" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="596" hidden="1">
+      <c r="A596" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>AD Halle</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D596" t="n">
+        <v>684</v>
+      </c>
+      <c r="E596" t="n">
+        <v>3</v>
+      </c>
+      <c r="F596" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H596" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I596" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="597" hidden="1">
+      <c r="A597" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>AD Bellegem</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D597" t="n">
+        <v>684</v>
+      </c>
+      <c r="E597" t="n">
+        <v>3</v>
+      </c>
+      <c r="F597" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H597" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I597" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="598" hidden="1">
+      <c r="A598" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>AD Watersport</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D598" t="n">
+        <v>684</v>
+      </c>
+      <c r="E598" t="n">
+        <v>3</v>
+      </c>
+      <c r="F598" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H598" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I598" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="599" hidden="1">
+      <c r="A599" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>AD ARENDONK</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D599" t="n">
+        <v>684</v>
+      </c>
+      <c r="E599" t="n">
+        <v>3</v>
+      </c>
+      <c r="F599" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H599" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I599" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="600" hidden="1">
+      <c r="A600" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>AD Retie</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D600" t="n">
+        <v>684</v>
+      </c>
+      <c r="E600" t="n">
+        <v>3</v>
+      </c>
+      <c r="F600" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H600" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I600" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="601" hidden="1">
+      <c r="A601" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>CM Square Marlow</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D601" t="n">
+        <v>684</v>
+      </c>
+      <c r="E601" t="n">
+        <v>3</v>
+      </c>
+      <c r="F601" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H601" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I601" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="602" hidden="1">
+      <c r="A602" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Fléron</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D602" t="n">
+        <v>684</v>
+      </c>
+      <c r="E602" t="n">
+        <v>3</v>
+      </c>
+      <c r="F602" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G602" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H602" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I602" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="603" hidden="1">
+      <c r="A603" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Cora Hornou</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D603" t="n">
+        <v>684</v>
+      </c>
+      <c r="E603" t="n">
+        <v>3</v>
+      </c>
+      <c r="F603" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H603" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I603" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="604" hidden="1">
+      <c r="A604" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Alma Geel</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D604" t="n">
+        <v>684</v>
+      </c>
+      <c r="E604" t="n">
+        <v>3</v>
+      </c>
+      <c r="F604" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G604" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H604" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I604" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="605" hidden="1">
+      <c r="A605" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Meeuwen</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D605" t="n">
+        <v>684</v>
+      </c>
+      <c r="E605" t="n">
+        <v>3</v>
+      </c>
+      <c r="F605" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G605" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H605" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I605" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="606" hidden="1">
+      <c r="A606" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>CM Alma Lommel</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D606" t="n">
+        <v>684</v>
+      </c>
+      <c r="E606" t="n">
+        <v>3</v>
+      </c>
+      <c r="F606" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H606" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I606" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="607" hidden="1">
+      <c r="A607" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>JUMBO 's Gravendeel van der Hoek</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D607" t="n">
+        <v>684</v>
+      </c>
+      <c r="E607" t="n">
+        <v>3</v>
+      </c>
+      <c r="F607" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G607" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H607" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I607" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="608" hidden="1">
+      <c r="A608" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>AD Denderleew</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D608" t="n">
+        <v>684</v>
+      </c>
+      <c r="E608" t="n">
+        <v>3</v>
+      </c>
+      <c r="F608" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H608" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I608" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="609" hidden="1">
+      <c r="A609" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Denderleew</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D609" t="n">
+        <v>684</v>
+      </c>
+      <c r="E609" t="n">
+        <v>3</v>
+      </c>
+      <c r="F609" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G609" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H609" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I609" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="610" hidden="1">
+      <c r="A610" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Merim Supermarket</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D610" t="n">
+        <v>684</v>
+      </c>
+      <c r="E610" t="n">
+        <v>3</v>
+      </c>
+      <c r="F610" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H610" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I610" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="611" hidden="1">
+      <c r="A611" t="n">
+        <v>8664</v>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>AH Roeselare</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="D611" t="n">
+        <v>684</v>
+      </c>
+      <c r="E611" t="n">
+        <v>3</v>
+      </c>
+      <c r="F611" s="201" t="n">
+        <v>45874</v>
+      </c>
+      <c r="G611" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H611" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I611" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="612" hidden="1">
+      <c r="A612" t="n">
+        <v>8665</v>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>AD Zottegem</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Y9</t>
+        </is>
+      </c>
+      <c r="D612" t="n">
+        <v>1368</v>
+      </c>
+      <c r="E612" t="n">
+        <v>6</v>
+      </c>
+      <c r="F612" s="201" t="n">
+        <v>46044</v>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H612" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I612" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="613" hidden="1">
+      <c r="A613" t="n">
+        <v>8665</v>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>AH Merksem MAATJES_x000D_</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Y9</t>
+        </is>
+      </c>
+      <c r="D613" t="n">
+        <v>1368</v>
+      </c>
+      <c r="E613" t="n">
+        <v>6</v>
+      </c>
+      <c r="F613" s="201" t="n">
+        <v>46044</v>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H613" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I613" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="614" hidden="1">
+      <c r="A614" t="n">
+        <v>8665</v>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>CM Alma Bilzen</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Y9</t>
+        </is>
+      </c>
+      <c r="D614" t="n">
+        <v>1368</v>
+      </c>
+      <c r="E614" t="n">
+        <v>6</v>
+      </c>
+      <c r="F614" s="201" t="n">
+        <v>46044</v>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H614" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I614" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="615" hidden="1">
+      <c r="A615" t="n">
+        <v>8665</v>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>AD Geraardsbergen_x000D_</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Y9</t>
+        </is>
+      </c>
+      <c r="D615" t="n">
+        <v>1368</v>
+      </c>
+      <c r="E615" t="n">
+        <v>6</v>
+      </c>
+      <c r="F615" s="201" t="n">
+        <v>46044</v>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H615" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I615" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="616" hidden="1">
+      <c r="A616" t="n">
+        <v>8665</v>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>AD Harelbeke</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Y9</t>
+        </is>
+      </c>
+      <c r="D616" t="n">
+        <v>1368</v>
+      </c>
+      <c r="E616" t="n">
+        <v>6</v>
+      </c>
+      <c r="F616" s="201" t="n">
+        <v>46044</v>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H616" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I616" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="617" hidden="1">
+      <c r="A617" t="n">
+        <v>8665</v>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>CM Alma mol</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Y9</t>
+        </is>
+      </c>
+      <c r="D617" t="n">
+        <v>1368</v>
+      </c>
+      <c r="E617" t="n">
+        <v>6</v>
+      </c>
+      <c r="F617" s="201" t="n">
+        <v>46044</v>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H617" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I617" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="618" hidden="1">
+      <c r="A618" t="n">
+        <v>8666</v>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>AD Zwevegem</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="D618" t="n">
+        <v>5016</v>
+      </c>
+      <c r="E618" t="n">
+        <v>22</v>
+      </c>
+      <c r="F618" s="201" t="n">
+        <v>46048</v>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H618" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I618" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="619" hidden="1">
+      <c r="A619" t="n">
+        <v>8666</v>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AD Deinze </t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="D619" t="n">
+        <v>5016</v>
+      </c>
+      <c r="E619" t="n">
+        <v>22</v>
+      </c>
+      <c r="F619" s="201" t="n">
+        <v>46048</v>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H619" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I619" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="620" hidden="1">
+      <c r="A620" t="n">
+        <v>8667</v>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="D620" t="n">
+        <v>684</v>
+      </c>
+      <c r="E620" t="n">
+        <v>3</v>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H620" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I620" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="621" hidden="1">
+      <c r="I621" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="622" hidden="1">
+      <c r="A622" t="n">
+        <v>8667</v>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AD Heist </t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="D622" t="n">
+        <v>684</v>
+      </c>
+      <c r="E622" t="n">
+        <v>3</v>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H622" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I622" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="623" hidden="1">
+      <c r="A623" t="n">
+        <v>8667</v>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>AD Waregem</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="D623" t="n">
+        <v>684</v>
+      </c>
+      <c r="E623" t="n">
+        <v>3</v>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H623" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I623" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="624" hidden="1">
+      <c r="A624" t="n">
+        <v>8667</v>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>AH Oudenaarde</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="D624" t="n">
+        <v>684</v>
+      </c>
+      <c r="E624" t="n">
+        <v>3</v>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H624" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I624" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="625" hidden="1">
+      <c r="A625" t="n">
+        <v>8667</v>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>AH Waregem</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="D625" t="n">
+        <v>684</v>
+      </c>
+      <c r="E625" t="n">
+        <v>3</v>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H625" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I625" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="626" hidden="1">
+      <c r="A626" t="n">
+        <v>8668</v>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>AD Wondelgem</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="D626" t="n">
+        <v>912</v>
+      </c>
+      <c r="E626" t="n">
+        <v>4</v>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H626" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I626" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="627" hidden="1">
+      <c r="A627" t="n">
+        <v>8668</v>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>CM Elouges</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="D627" t="n">
+        <v>912</v>
+      </c>
+      <c r="E627" t="n">
+        <v>4</v>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H627" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I627" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="628" hidden="1">
+      <c r="A628" t="n">
+        <v>8668</v>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>CM St-Gillis-Waas</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="D628" t="n">
+        <v>912</v>
+      </c>
+      <c r="E628" t="n">
+        <v>4</v>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H628" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I628" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="629" hidden="1">
+      <c r="A629" t="n">
+        <v>8668</v>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Muizen</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="D629" t="n">
+        <v>912</v>
+      </c>
+      <c r="E629" t="n">
+        <v>4</v>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H629" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I629" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="630" hidden="1">
+      <c r="A630" t="n">
+        <v>8668</v>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Proxy Delhaize Denderhoutem</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="D630" t="n">
+        <v>912</v>
+      </c>
+      <c r="E630" t="n">
+        <v>4</v>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H630" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I630" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="631" hidden="1">
+      <c r="A631" t="n">
+        <v>8668</v>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proxy Delhaize Grootzand </t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="D631" t="n">
+        <v>912</v>
+      </c>
+      <c r="E631" t="n">
+        <v>4</v>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H631" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I631" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="632" hidden="1">
+      <c r="A632" t="n">
+        <v>8668</v>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>AD Zwijnaarde</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="D632" t="n">
+        <v>912</v>
+      </c>
+      <c r="E632" t="n">
+        <v>4</v>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H632" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I632" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="633" hidden="1">
+      <c r="A633" t="n">
+        <v>8668</v>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AH Schilde </t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="D633" t="n">
+        <v>912</v>
+      </c>
+      <c r="E633" t="n">
+        <v>4</v>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H633" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I633" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="n">
+        <v>8668</v>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>CM Oedelem</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="D634" t="n">
+        <v>912</v>
+      </c>
+      <c r="E634" t="n">
+        <v>4</v>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H634" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I634" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>AD Delhaize Sint Lenaarts</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D635" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E635" t="n">
+        <v>10</v>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H635" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I635" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>AD Delhaize Fernelmont</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D636" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E636" t="n">
+        <v>10</v>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H636" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I636" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Proxy Delhaize OOIGEM</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D637" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E637" t="n">
+        <v>10</v>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H637" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I637" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Proxy Delhaize Wakken</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D638" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E638" t="n">
+        <v>10</v>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H638" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I638" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="n">
+        <v>8670</v>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>intermarché Heusy</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="D639" t="n">
+        <v>7780</v>
+      </c>
+      <c r="E639" t="n">
+        <v>10</v>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H639" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I639" t="n">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="n">
+        <v>8669</v>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Rewe Schorn - Bergheim</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Paid Trial-0.5Y</t>
+        </is>
+      </c>
+      <c r="D640" t="n">
+        <v>389</v>
+      </c>
+      <c r="E640" t="n">
+        <v>1</v>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H640" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="n">
+        <v>8669</v>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Edeka Kusnezow-Lewandowski - Langerwehe</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Paid Trial-0.5Y</t>
+        </is>
+      </c>
+      <c r="D641" t="n">
+        <v>389</v>
+      </c>
+      <c r="E641" t="n">
+        <v>1</v>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H641" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="n">
+        <v>8669</v>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Edeka Vogel-Lewandowski - Dueren</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Paid Trial-0.5Y</t>
+        </is>
+      </c>
+      <c r="D642" t="n">
+        <v>389</v>
+      </c>
+      <c r="E642" t="n">
+        <v>1</v>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H642" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="n">
+        <v>8669</v>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Edeka Vogel - Dueren</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Paid Trial-0.5Y</t>
+        </is>
+      </c>
+      <c r="D643" t="n">
+        <v>389</v>
+      </c>
+      <c r="E643" t="n">
+        <v>1</v>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H643" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="n">
+        <v>8669</v>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Edeka Billstein - Wuppertal</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Paid Trial-0.5Y</t>
+        </is>
+      </c>
+      <c r="D644" t="n">
+        <v>389</v>
+      </c>
+      <c r="E644" t="n">
+        <v>1</v>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H644" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="n">
+        <v>8669</v>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Edeka Hoevener - Langenfeld</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Paid Trial-0.5Y</t>
+        </is>
+      </c>
+      <c r="D645" t="n">
+        <v>389</v>
+      </c>
+      <c r="E645" t="n">
+        <v>1</v>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H645" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="n">
+        <v>8669</v>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Edeka Paschmann - Muelheim</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Paid Trial-0.5Y</t>
+        </is>
+      </c>
+      <c r="D646" t="n">
+        <v>389</v>
+      </c>
+      <c r="E646" t="n">
+        <v>1</v>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H646" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="n">
+        <v>8669</v>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Edeka Steren - Sulingen</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Paid Trial-0.5Y</t>
+        </is>
+      </c>
+      <c r="D647" t="n">
+        <v>389</v>
+      </c>
+      <c r="E647" t="n">
+        <v>1</v>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H647" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="n">
+        <v>8669</v>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Edeka Rath - Grevenbroich</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Paid Trial-0.5Y</t>
+        </is>
+      </c>
+      <c r="D648" t="n">
+        <v>389</v>
+      </c>
+      <c r="E648" t="n">
+        <v>1</v>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H648" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="n">
+        <v>8671</v>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>CM Meer</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>M-7Y</t>
+        </is>
+      </c>
+      <c r="D649" t="n">
+        <v>684</v>
+      </c>
+      <c r="E649" t="n">
+        <v>3</v>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H649" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="n">
+        <v>8671</v>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>AH Ninove</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>M-7Y</t>
+        </is>
+      </c>
+      <c r="D650" t="n">
+        <v>684</v>
+      </c>
+      <c r="E650" t="n">
+        <v>3</v>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H650" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="n">
+        <v>8671</v>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>AH Dendermonde</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>M-7Y</t>
+        </is>
+      </c>
+      <c r="D651" t="n">
+        <v>684</v>
+      </c>
+      <c r="E651" t="n">
+        <v>3</v>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H651" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="n">
+        <v>8671</v>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>AH Rumbeke</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>M-7Y</t>
+        </is>
+      </c>
+      <c r="D652" t="n">
+        <v>684</v>
+      </c>
+      <c r="E652" t="n">
+        <v>3</v>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H652" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="n">
+        <v>8671</v>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>CM Sint-Niklaas</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>M-7Y</t>
+        </is>
+      </c>
+      <c r="D653" t="n">
+        <v>684</v>
+      </c>
+      <c r="E653" t="n">
+        <v>3</v>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H653" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="n">
+        <v>8671</v>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>CM Zeebrugge</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>M-7Y</t>
+        </is>
+      </c>
+      <c r="D654" t="n">
+        <v>684</v>
+      </c>
+      <c r="E654" t="n">
+        <v>3</v>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H654" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="n">
+        <v>8672</v>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>CM Hoboken Zuid</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>M-2Y</t>
+        </is>
+      </c>
+      <c r="D655" t="n">
+        <v>684</v>
+      </c>
+      <c r="E655" t="n">
+        <v>3</v>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H655" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="n">
+        <v>8672</v>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>CM Hoboken Kiosk</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>M-2Y</t>
+        </is>
+      </c>
+      <c r="D656" t="n">
+        <v>684</v>
+      </c>
+      <c r="E656" t="n">
+        <v>3</v>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H656" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="n">
+        <v>8672</v>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>AD Heist-op-den-Berg</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>M-2Y</t>
+        </is>
+      </c>
+      <c r="D657" t="n">
+        <v>684</v>
+      </c>
+      <c r="E657" t="n">
+        <v>3</v>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H657" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="n">
+        <v>8672</v>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>AD Brecht</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>M-2Y</t>
+        </is>
+      </c>
+      <c r="D658" t="n">
+        <v>684</v>
+      </c>
+      <c r="E658" t="n">
+        <v>3</v>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H658" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="n">
+        <v>8672</v>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>AD Merksplas</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>M-2Y</t>
+        </is>
+      </c>
+      <c r="D659" t="n">
+        <v>684</v>
+      </c>
+      <c r="E659" t="n">
+        <v>3</v>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H659" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="n">
+        <v>8672</v>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>AD GrootBijgaarden</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>M-2Y</t>
+        </is>
+      </c>
+      <c r="D660" t="n">
+        <v>684</v>
+      </c>
+      <c r="E660" t="n">
+        <v>3</v>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H660" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="661" ht="101.25" customHeight="1">
+      <c r="A661" t="n">
+        <v>8672</v>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>AD Vichte</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>M-2Y</t>
+        </is>
+      </c>
+      <c r="D661" t="n">
+        <v>684</v>
+      </c>
+      <c r="E661" t="n">
+        <v>3</v>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H661" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="n">
+        <v>8672</v>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>PLUS Simpelveld Schouteten</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>M-2Y</t>
+        </is>
+      </c>
+      <c r="D662" t="n">
+        <v>684</v>
+      </c>
+      <c r="E662" t="n">
+        <v>3</v>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H662" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="n">
+        <v>8672</v>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>JUMBO Eindhoven Boschdijk</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>M-2Y</t>
+        </is>
+      </c>
+      <c r="D663" t="n">
+        <v>684</v>
+      </c>
+      <c r="E663" t="n">
+        <v>3</v>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H663" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="n">
         <v>8673</v>
       </c>
-      <c r="B560" t="inlineStr">
+      <c r="B664" t="inlineStr">
         <is>
           <t>AD Anderlecht</t>
         </is>
       </c>
-      <c r="C560" t="inlineStr">
+      <c r="C664" t="inlineStr">
         <is>
           <t>M-1Y</t>
         </is>
       </c>
-      <c r="D560" t="n">
+      <c r="D664" t="n">
         <v>1556</v>
       </c>
-      <c r="E560" t="n">
+      <c r="E664" t="n">
         <v>2</v>
       </c>
-      <c r="G560" t="inlineStr">
+      <c r="G664" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H560" t="n">
+      <c r="H664" t="n">
         <v>2026</v>
       </c>
     </row>
-    <row r="561" hidden="1"/>
-    <row r="562" hidden="1"/>
-    <row r="563" hidden="1"/>
-    <row r="564" hidden="1"/>
-    <row r="565" hidden="1"/>
-    <row r="566" hidden="1"/>
-    <row r="567" hidden="1"/>
-    <row r="568" hidden="1"/>
-    <row r="569" hidden="1"/>
-    <row r="570" hidden="1"/>
-    <row r="571" hidden="1"/>
-    <row r="572" hidden="1"/>
-    <row r="573" hidden="1"/>
-    <row r="574" hidden="1"/>
-    <row r="575" hidden="1"/>
-    <row r="576" hidden="1"/>
-    <row r="577" hidden="1"/>
-    <row r="578" hidden="1"/>
-    <row r="579" hidden="1"/>
-    <row r="580" hidden="1"/>
-    <row r="581" hidden="1"/>
-    <row r="582" hidden="1"/>
-    <row r="583" hidden="1"/>
-    <row r="584" hidden="1"/>
-    <row r="585" hidden="1"/>
-    <row r="586" hidden="1"/>
-    <row r="587" hidden="1"/>
-    <row r="588" hidden="1"/>
-    <row r="589" hidden="1"/>
-    <row r="590" hidden="1"/>
-    <row r="591" hidden="1"/>
-    <row r="592" hidden="1"/>
-    <row r="593" hidden="1"/>
-    <row r="594" hidden="1"/>
-    <row r="595" hidden="1"/>
-    <row r="596" hidden="1"/>
-    <row r="597" hidden="1"/>
-    <row r="598" hidden="1"/>
-    <row r="599" hidden="1"/>
-    <row r="600" hidden="1"/>
-    <row r="601" hidden="1"/>
-    <row r="602" hidden="1"/>
-    <row r="603" hidden="1"/>
-    <row r="604" hidden="1"/>
-    <row r="605" hidden="1"/>
-    <row r="606" hidden="1"/>
-    <row r="607" hidden="1"/>
-    <row r="608" hidden="1"/>
-    <row r="609" hidden="1"/>
-    <row r="610" hidden="1"/>
-    <row r="611" hidden="1"/>
-    <row r="612" hidden="1"/>
-    <row r="613" hidden="1"/>
-    <row r="614" hidden="1"/>
-    <row r="615" hidden="1"/>
-    <row r="616" hidden="1"/>
-    <row r="617" hidden="1"/>
-    <row r="618" hidden="1"/>
-    <row r="619" hidden="1"/>
-    <row r="620" hidden="1"/>
-    <row r="621" hidden="1"/>
-    <row r="622" hidden="1"/>
-    <row r="623" hidden="1"/>
-    <row r="624" hidden="1"/>
-    <row r="625" hidden="1"/>
-    <row r="626" hidden="1"/>
-    <row r="627" hidden="1"/>
-    <row r="628" hidden="1"/>
-    <row r="629" hidden="1"/>
-    <row r="630" hidden="1"/>
-    <row r="631" hidden="1"/>
-    <row r="632" hidden="1"/>
-    <row r="633" hidden="1"/>
-    <row r="661" ht="101.25" customHeight="1"/>
+    <row r="665">
+      <c r="A665" t="n">
+        <v>8673</v>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>AD Burenvile</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>M-1Y</t>
+        </is>
+      </c>
+      <c r="D665" t="n">
+        <v>1556</v>
+      </c>
+      <c r="E665" t="n">
+        <v>2</v>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H665" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="n">
+        <v>8673</v>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>EDEKA DORTMUND</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>M-1Y</t>
+        </is>
+      </c>
+      <c r="D666" t="n">
+        <v>1556</v>
+      </c>
+      <c r="E666" t="n">
+        <v>2</v>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H666" t="n">
+        <v>2026</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I670">
     <filterColumn colId="2" hiddenButton="0" showButton="1">

</xml_diff>

<commit_message>
Fix invoice 8670 camera counts and amounts from PDF
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -37483,10 +37483,10 @@
         </is>
       </c>
       <c r="D550" t="n">
-        <v>7780</v>
+        <v>9336</v>
       </c>
       <c r="E550" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G550" t="inlineStr">
         <is>
@@ -37547,10 +37547,10 @@
         </is>
       </c>
       <c r="D552" t="n">
-        <v>7780</v>
+        <v>3112</v>
       </c>
       <c r="E552" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G552" t="inlineStr">
         <is>
@@ -37579,10 +37579,10 @@
         </is>
       </c>
       <c r="D553" t="n">
-        <v>7780</v>
+        <v>10892</v>
       </c>
       <c r="E553" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G553" t="inlineStr">
         <is>
@@ -37611,10 +37611,10 @@
         </is>
       </c>
       <c r="D554" t="n">
-        <v>7780</v>
+        <v>6224</v>
       </c>
       <c r="E554" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G554" t="inlineStr">
         <is>
@@ -37643,10 +37643,10 @@
         </is>
       </c>
       <c r="D555" t="n">
-        <v>7780</v>
+        <v>12448</v>
       </c>
       <c r="E555" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G555" t="inlineStr">
         <is>
@@ -37675,10 +37675,10 @@
         </is>
       </c>
       <c r="D556" t="n">
-        <v>7780</v>
+        <v>7002</v>
       </c>
       <c r="E556" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G556" t="inlineStr">
         <is>
@@ -37707,10 +37707,10 @@
         </is>
       </c>
       <c r="D557" t="n">
-        <v>7780</v>
+        <v>12448</v>
       </c>
       <c r="E557" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G557" t="inlineStr">
         <is>
@@ -37739,10 +37739,10 @@
         </is>
       </c>
       <c r="D558" t="n">
-        <v>7780</v>
+        <v>6224</v>
       </c>
       <c r="E558" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G558" t="inlineStr">
         <is>
@@ -37771,10 +37771,10 @@
         </is>
       </c>
       <c r="D559" t="n">
-        <v>7780</v>
+        <v>12448</v>
       </c>
       <c r="E559" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G559" t="inlineStr">
         <is>
@@ -37803,10 +37803,10 @@
         </is>
       </c>
       <c r="D560" t="n">
-        <v>7780</v>
+        <v>4668</v>
       </c>
       <c r="E560" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G560" t="inlineStr">
         <is>
@@ -37835,10 +37835,10 @@
         </is>
       </c>
       <c r="D561" t="n">
-        <v>7780</v>
+        <v>6224</v>
       </c>
       <c r="E561" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G561" t="inlineStr">
         <is>
@@ -37867,10 +37867,10 @@
         </is>
       </c>
       <c r="D562" t="n">
-        <v>7780</v>
+        <v>9336</v>
       </c>
       <c r="E562" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G562" t="inlineStr">
         <is>
@@ -37899,10 +37899,10 @@
         </is>
       </c>
       <c r="D563" t="n">
-        <v>7780</v>
+        <v>9336</v>
       </c>
       <c r="E563" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G563" t="inlineStr">
         <is>
@@ -37931,10 +37931,10 @@
         </is>
       </c>
       <c r="D564" t="n">
-        <v>7780</v>
+        <v>6224</v>
       </c>
       <c r="E564" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G564" t="inlineStr">
         <is>
@@ -37963,10 +37963,10 @@
         </is>
       </c>
       <c r="D565" t="n">
-        <v>7780</v>
+        <v>6224</v>
       </c>
       <c r="E565" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G565" t="inlineStr">
         <is>
@@ -37995,10 +37995,10 @@
         </is>
       </c>
       <c r="D566" t="n">
-        <v>7780</v>
+        <v>1556</v>
       </c>
       <c r="E566" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G566" t="inlineStr">
         <is>
@@ -40319,10 +40319,10 @@
         </is>
       </c>
       <c r="D635" t="n">
-        <v>7780</v>
+        <v>6224</v>
       </c>
       <c r="E635" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G635" t="inlineStr">
         <is>
@@ -40351,10 +40351,10 @@
         </is>
       </c>
       <c r="D636" t="n">
-        <v>7780</v>
+        <v>6224</v>
       </c>
       <c r="E636" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G636" t="inlineStr">
         <is>
@@ -40383,10 +40383,10 @@
         </is>
       </c>
       <c r="D637" t="n">
-        <v>7780</v>
+        <v>6224</v>
       </c>
       <c r="E637" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G637" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix camera counts for invoices 8664-8673 from PDFs
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -38062,10 +38062,10 @@
         </is>
       </c>
       <c r="D568" t="n">
-        <v>684</v>
+        <v>5016</v>
       </c>
       <c r="E568" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="F568" s="201" t="n">
         <v>45874</v>
@@ -38097,10 +38097,10 @@
         </is>
       </c>
       <c r="D569" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E569" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F569" s="201" t="n">
         <v>45874</v>
@@ -38132,10 +38132,10 @@
         </is>
       </c>
       <c r="D570" t="n">
-        <v>684</v>
+        <v>1368</v>
       </c>
       <c r="E570" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F570" s="201" t="n">
         <v>45874</v>
@@ -38167,10 +38167,10 @@
         </is>
       </c>
       <c r="D571" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E571" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F571" s="201" t="n">
         <v>45874</v>
@@ -38202,10 +38202,10 @@
         </is>
       </c>
       <c r="D572" t="n">
-        <v>684</v>
+        <v>2736</v>
       </c>
       <c r="E572" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F572" s="201" t="n">
         <v>45874</v>
@@ -38237,10 +38237,10 @@
         </is>
       </c>
       <c r="D573" t="n">
-        <v>684</v>
+        <v>3192</v>
       </c>
       <c r="E573" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="F573" s="201" t="n">
         <v>45874</v>
@@ -38272,10 +38272,10 @@
         </is>
       </c>
       <c r="D574" t="n">
-        <v>684</v>
+        <v>3192</v>
       </c>
       <c r="E574" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="F574" s="201" t="n">
         <v>45874</v>
@@ -38307,10 +38307,10 @@
         </is>
       </c>
       <c r="D575" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E575" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F575" s="201" t="n">
         <v>45874</v>
@@ -38412,10 +38412,10 @@
         </is>
       </c>
       <c r="D578" t="n">
-        <v>684</v>
+        <v>2280</v>
       </c>
       <c r="E578" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F578" s="201" t="n">
         <v>45874</v>
@@ -38447,10 +38447,10 @@
         </is>
       </c>
       <c r="D579" t="n">
-        <v>684</v>
+        <v>1368</v>
       </c>
       <c r="E579" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F579" s="201" t="n">
         <v>45874</v>
@@ -38482,10 +38482,10 @@
         </is>
       </c>
       <c r="D580" t="n">
-        <v>684</v>
+        <v>2736</v>
       </c>
       <c r="E580" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F580" s="201" t="n">
         <v>45874</v>
@@ -38517,10 +38517,10 @@
         </is>
       </c>
       <c r="D581" t="n">
-        <v>684</v>
+        <v>5928</v>
       </c>
       <c r="E581" t="n">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="F581" s="201" t="n">
         <v>45874</v>
@@ -38552,10 +38552,10 @@
         </is>
       </c>
       <c r="D582" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E582" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F582" s="201" t="n">
         <v>45874</v>
@@ -38587,10 +38587,10 @@
         </is>
       </c>
       <c r="D583" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E583" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F583" s="201" t="n">
         <v>45874</v>
@@ -38622,10 +38622,10 @@
         </is>
       </c>
       <c r="D584" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E584" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F584" s="201" t="n">
         <v>45874</v>
@@ -38657,10 +38657,10 @@
         </is>
       </c>
       <c r="D585" t="n">
-        <v>684</v>
+        <v>4104</v>
       </c>
       <c r="E585" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="F585" s="201" t="n">
         <v>45874</v>
@@ -38692,10 +38692,10 @@
         </is>
       </c>
       <c r="D586" t="n">
-        <v>684</v>
+        <v>1368</v>
       </c>
       <c r="E586" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F586" s="201" t="n">
         <v>45874</v>
@@ -38727,10 +38727,10 @@
         </is>
       </c>
       <c r="D587" t="n">
-        <v>684</v>
+        <v>1140</v>
       </c>
       <c r="E587" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F587" s="201" t="n">
         <v>45874</v>
@@ -38797,10 +38797,10 @@
         </is>
       </c>
       <c r="D589" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E589" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F589" s="201" t="n">
         <v>45874</v>
@@ -38832,10 +38832,10 @@
         </is>
       </c>
       <c r="D590" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E590" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F590" s="201" t="n">
         <v>45874</v>
@@ -38867,10 +38867,10 @@
         </is>
       </c>
       <c r="D591" t="n">
-        <v>684</v>
+        <v>1368</v>
       </c>
       <c r="E591" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F591" s="201" t="n">
         <v>45874</v>
@@ -38926,10 +38926,10 @@
         </is>
       </c>
       <c r="D593" t="n">
-        <v>684</v>
+        <v>2280</v>
       </c>
       <c r="E593" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F593" s="201" t="n">
         <v>45874</v>
@@ -38961,10 +38961,10 @@
         </is>
       </c>
       <c r="D594" t="n">
-        <v>684</v>
+        <v>2964</v>
       </c>
       <c r="E594" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="F594" s="201" t="n">
         <v>45874</v>
@@ -38996,10 +38996,10 @@
         </is>
       </c>
       <c r="D595" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E595" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F595" s="201" t="n">
         <v>45874</v>
@@ -39031,10 +39031,10 @@
         </is>
       </c>
       <c r="D596" t="n">
-        <v>684</v>
+        <v>3192</v>
       </c>
       <c r="E596" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="F596" s="201" t="n">
         <v>45874</v>
@@ -39066,10 +39066,10 @@
         </is>
       </c>
       <c r="D597" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E597" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F597" s="201" t="n">
         <v>45874</v>
@@ -39101,10 +39101,10 @@
         </is>
       </c>
       <c r="D598" t="n">
-        <v>684</v>
+        <v>3648</v>
       </c>
       <c r="E598" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="F598" s="201" t="n">
         <v>45874</v>
@@ -39136,10 +39136,10 @@
         </is>
       </c>
       <c r="D599" t="n">
-        <v>684</v>
+        <v>2280</v>
       </c>
       <c r="E599" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F599" s="201" t="n">
         <v>45874</v>
@@ -39171,10 +39171,10 @@
         </is>
       </c>
       <c r="D600" t="n">
-        <v>684</v>
+        <v>2736</v>
       </c>
       <c r="E600" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F600" s="201" t="n">
         <v>45874</v>
@@ -39206,10 +39206,10 @@
         </is>
       </c>
       <c r="D601" t="n">
-        <v>684</v>
+        <v>1368</v>
       </c>
       <c r="E601" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F601" s="201" t="n">
         <v>45874</v>
@@ -39241,10 +39241,10 @@
         </is>
       </c>
       <c r="D602" t="n">
-        <v>684</v>
+        <v>2280</v>
       </c>
       <c r="E602" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F602" s="201" t="n">
         <v>45874</v>
@@ -39276,10 +39276,10 @@
         </is>
       </c>
       <c r="D603" t="n">
-        <v>684</v>
+        <v>2736</v>
       </c>
       <c r="E603" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F603" s="201" t="n">
         <v>45874</v>
@@ -39311,10 +39311,10 @@
         </is>
       </c>
       <c r="D604" t="n">
-        <v>684</v>
+        <v>1368</v>
       </c>
       <c r="E604" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F604" s="201" t="n">
         <v>45874</v>
@@ -39346,10 +39346,10 @@
         </is>
       </c>
       <c r="D605" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E605" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F605" s="201" t="n">
         <v>45874</v>
@@ -39381,10 +39381,10 @@
         </is>
       </c>
       <c r="D606" t="n">
-        <v>684</v>
+        <v>912</v>
       </c>
       <c r="E606" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F606" s="201" t="n">
         <v>45874</v>
@@ -39521,10 +39521,10 @@
         </is>
       </c>
       <c r="D610" t="n">
-        <v>684</v>
+        <v>2280</v>
       </c>
       <c r="E610" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F610" s="201" t="n">
         <v>45874</v>
@@ -39591,10 +39591,10 @@
         </is>
       </c>
       <c r="D612" t="n">
-        <v>1368</v>
+        <v>2736</v>
       </c>
       <c r="E612" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F612" s="201" t="n">
         <v>46044</v>
@@ -39661,10 +39661,10 @@
         </is>
       </c>
       <c r="D614" t="n">
-        <v>1368</v>
+        <v>912</v>
       </c>
       <c r="E614" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F614" s="201" t="n">
         <v>46044</v>
@@ -39731,10 +39731,10 @@
         </is>
       </c>
       <c r="D616" t="n">
-        <v>1368</v>
+        <v>3648</v>
       </c>
       <c r="E616" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F616" s="201" t="n">
         <v>46044</v>
@@ -39801,10 +39801,10 @@
         </is>
       </c>
       <c r="D618" t="n">
-        <v>5016</v>
+        <v>3192</v>
       </c>
       <c r="E618" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F618" s="201" t="n">
         <v>46048</v>
@@ -39903,10 +39903,10 @@
         </is>
       </c>
       <c r="D622" t="n">
-        <v>684</v>
+        <v>4104</v>
       </c>
       <c r="E622" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="G622" t="inlineStr">
         <is>
@@ -39935,10 +39935,10 @@
         </is>
       </c>
       <c r="D623" t="n">
-        <v>684</v>
+        <v>4560</v>
       </c>
       <c r="E623" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="G623" t="inlineStr">
         <is>
@@ -40031,10 +40031,10 @@
         </is>
       </c>
       <c r="D626" t="n">
-        <v>912</v>
+        <v>2736</v>
       </c>
       <c r="E626" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G626" t="inlineStr">
         <is>
@@ -40095,10 +40095,10 @@
         </is>
       </c>
       <c r="D628" t="n">
-        <v>912</v>
+        <v>1140</v>
       </c>
       <c r="E628" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G628" t="inlineStr">
         <is>
@@ -40127,10 +40127,10 @@
         </is>
       </c>
       <c r="D629" t="n">
-        <v>912</v>
+        <v>1824</v>
       </c>
       <c r="E629" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G629" t="inlineStr">
         <is>
@@ -40191,10 +40191,10 @@
         </is>
       </c>
       <c r="D631" t="n">
-        <v>912</v>
+        <v>2280</v>
       </c>
       <c r="E631" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G631" t="inlineStr">
         <is>
@@ -40223,10 +40223,10 @@
         </is>
       </c>
       <c r="D632" t="n">
-        <v>912</v>
+        <v>1596</v>
       </c>
       <c r="E632" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G632" t="inlineStr">
         <is>
@@ -40740,10 +40740,10 @@
         </is>
       </c>
       <c r="D649" t="n">
-        <v>684</v>
+        <v>1368</v>
       </c>
       <c r="E649" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G649" t="inlineStr">
         <is>
@@ -40769,10 +40769,10 @@
         </is>
       </c>
       <c r="D650" t="n">
-        <v>684</v>
+        <v>912</v>
       </c>
       <c r="E650" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G650" t="inlineStr">
         <is>
@@ -40798,10 +40798,10 @@
         </is>
       </c>
       <c r="D651" t="n">
-        <v>684</v>
+        <v>912</v>
       </c>
       <c r="E651" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G651" t="inlineStr">
         <is>
@@ -40827,10 +40827,10 @@
         </is>
       </c>
       <c r="D652" t="n">
-        <v>684</v>
+        <v>912</v>
       </c>
       <c r="E652" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G652" t="inlineStr">
         <is>
@@ -40856,10 +40856,10 @@
         </is>
       </c>
       <c r="D653" t="n">
-        <v>684</v>
+        <v>1596</v>
       </c>
       <c r="E653" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G653" t="inlineStr">
         <is>
@@ -40914,10 +40914,10 @@
         </is>
       </c>
       <c r="D655" t="n">
-        <v>684</v>
+        <v>2736</v>
       </c>
       <c r="E655" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G655" t="inlineStr">
         <is>
@@ -40943,10 +40943,10 @@
         </is>
       </c>
       <c r="D656" t="n">
-        <v>684</v>
+        <v>2280</v>
       </c>
       <c r="E656" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G656" t="inlineStr">
         <is>
@@ -40972,10 +40972,10 @@
         </is>
       </c>
       <c r="D657" t="n">
-        <v>684</v>
+        <v>2280</v>
       </c>
       <c r="E657" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G657" t="inlineStr">
         <is>
@@ -41001,10 +41001,10 @@
         </is>
       </c>
       <c r="D658" t="n">
-        <v>684</v>
+        <v>2736</v>
       </c>
       <c r="E658" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G658" t="inlineStr">
         <is>
@@ -41059,10 +41059,10 @@
         </is>
       </c>
       <c r="D660" t="n">
-        <v>684</v>
+        <v>4560</v>
       </c>
       <c r="E660" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="G660" t="inlineStr">
         <is>
@@ -41088,10 +41088,10 @@
         </is>
       </c>
       <c r="D661" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E661" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G661" t="inlineStr">
         <is>
@@ -41175,10 +41175,10 @@
         </is>
       </c>
       <c r="D664" t="n">
-        <v>1556</v>
+        <v>4668</v>
       </c>
       <c r="E664" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G664" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix remaining camera count mismatches from PDFs
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -38342,10 +38342,10 @@
         </is>
       </c>
       <c r="D576" t="n">
-        <v>684</v>
+        <v>1368</v>
       </c>
       <c r="E576" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F576" s="201" t="n">
         <v>45874</v>
@@ -38377,10 +38377,10 @@
         </is>
       </c>
       <c r="D577" t="n">
-        <v>684</v>
+        <v>1368</v>
       </c>
       <c r="E577" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F577" s="201" t="n">
         <v>45874</v>
@@ -38762,10 +38762,10 @@
         </is>
       </c>
       <c r="D588" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E588" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F588" s="201" t="n">
         <v>45874</v>
@@ -39451,10 +39451,10 @@
         </is>
       </c>
       <c r="D608" t="n">
-        <v>684</v>
+        <v>2736</v>
       </c>
       <c r="E608" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F608" s="201" t="n">
         <v>45874</v>
@@ -39486,10 +39486,10 @@
         </is>
       </c>
       <c r="D609" t="n">
-        <v>684</v>
+        <v>1140</v>
       </c>
       <c r="E609" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F609" s="201" t="n">
         <v>45874</v>
@@ -39626,10 +39626,10 @@
         </is>
       </c>
       <c r="D613" t="n">
-        <v>1368</v>
+        <v>912</v>
       </c>
       <c r="E613" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F613" s="201" t="n">
         <v>46044</v>
@@ -39696,10 +39696,10 @@
         </is>
       </c>
       <c r="D615" t="n">
-        <v>1368</v>
+        <v>1140</v>
       </c>
       <c r="E615" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F615" s="201" t="n">
         <v>46044</v>
@@ -40415,10 +40415,10 @@
         </is>
       </c>
       <c r="D638" t="n">
-        <v>7780</v>
+        <v>6224</v>
       </c>
       <c r="E638" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G638" t="inlineStr">
         <is>
@@ -41030,10 +41030,10 @@
         </is>
       </c>
       <c r="D659" t="n">
-        <v>684</v>
+        <v>1824</v>
       </c>
       <c r="E659" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G659" t="inlineStr">
         <is>
@@ -41117,10 +41117,10 @@
         </is>
       </c>
       <c r="D662" t="n">
-        <v>684</v>
+        <v>1140</v>
       </c>
       <c r="E662" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G662" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Standardize project name variants in Invoice details
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -19417,7 +19417,7 @@
     <row r="132">
       <c r="A132" s="73" t="inlineStr">
         <is>
-          <t>PLUS Simpelveld Schouteten</t>
+          <t>Plus Simpelveld Schouteten</t>
         </is>
       </c>
       <c r="B132" s="31" t="inlineStr">
@@ -19541,12 +19541,446 @@
         <v>46388</v>
       </c>
     </row>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
     <row r="180">
       <c r="J180" s="92" t="n"/>
     </row>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
     <row r="184">
       <c r="J184" s="78" t="n"/>
     </row>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
+    <row r="212"/>
+    <row r="213"/>
+    <row r="214"/>
+    <row r="215"/>
+    <row r="216"/>
+    <row r="217"/>
+    <row r="218"/>
+    <row r="219"/>
+    <row r="220"/>
+    <row r="221"/>
+    <row r="222"/>
+    <row r="223"/>
+    <row r="224"/>
+    <row r="225"/>
+    <row r="226"/>
+    <row r="227"/>
+    <row r="228"/>
+    <row r="229"/>
+    <row r="230"/>
+    <row r="231"/>
+    <row r="232"/>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
+    <row r="281"/>
+    <row r="282"/>
+    <row r="283"/>
+    <row r="284"/>
+    <row r="285"/>
+    <row r="286"/>
+    <row r="287"/>
+    <row r="288"/>
+    <row r="289"/>
+    <row r="290"/>
+    <row r="291"/>
+    <row r="292"/>
+    <row r="293"/>
+    <row r="294"/>
+    <row r="295"/>
+    <row r="296"/>
+    <row r="297"/>
+    <row r="298"/>
+    <row r="299"/>
+    <row r="300"/>
+    <row r="301"/>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304"/>
+    <row r="305"/>
+    <row r="306"/>
+    <row r="307"/>
+    <row r="308"/>
+    <row r="309"/>
+    <row r="310"/>
+    <row r="311"/>
+    <row r="312"/>
+    <row r="313"/>
+    <row r="314"/>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317"/>
+    <row r="318"/>
+    <row r="319"/>
+    <row r="320"/>
+    <row r="321"/>
+    <row r="322"/>
+    <row r="323"/>
+    <row r="324"/>
+    <row r="325"/>
+    <row r="326"/>
+    <row r="327"/>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330"/>
+    <row r="331"/>
+    <row r="332"/>
+    <row r="333"/>
+    <row r="334"/>
+    <row r="335"/>
+    <row r="336"/>
+    <row r="337"/>
+    <row r="338"/>
+    <row r="339"/>
+    <row r="340"/>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343"/>
+    <row r="344"/>
+    <row r="345"/>
+    <row r="346"/>
+    <row r="347"/>
+    <row r="348"/>
+    <row r="349"/>
+    <row r="350"/>
+    <row r="351"/>
+    <row r="352"/>
+    <row r="353"/>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356"/>
+    <row r="357"/>
+    <row r="358"/>
+    <row r="359"/>
+    <row r="360"/>
+    <row r="361"/>
+    <row r="362"/>
+    <row r="363"/>
+    <row r="364"/>
+    <row r="365"/>
+    <row r="366"/>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369"/>
+    <row r="370"/>
+    <row r="371"/>
+    <row r="372"/>
+    <row r="373"/>
+    <row r="374"/>
+    <row r="375"/>
+    <row r="376"/>
+    <row r="377"/>
+    <row r="378"/>
+    <row r="379"/>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
+    <row r="383"/>
+    <row r="384"/>
+    <row r="385"/>
+    <row r="386"/>
+    <row r="387"/>
+    <row r="388"/>
+    <row r="389"/>
+    <row r="390"/>
+    <row r="391"/>
+    <row r="392"/>
+    <row r="393"/>
+    <row r="394"/>
+    <row r="395"/>
+    <row r="396"/>
+    <row r="397"/>
+    <row r="398"/>
+    <row r="399"/>
+    <row r="400"/>
+    <row r="401"/>
+    <row r="402"/>
+    <row r="403"/>
+    <row r="404"/>
+    <row r="405"/>
+    <row r="406"/>
+    <row r="407"/>
+    <row r="408"/>
+    <row r="409"/>
+    <row r="410"/>
+    <row r="411"/>
+    <row r="412"/>
+    <row r="413"/>
+    <row r="414"/>
+    <row r="415"/>
+    <row r="416"/>
+    <row r="417"/>
+    <row r="418"/>
+    <row r="419"/>
+    <row r="420"/>
+    <row r="421"/>
+    <row r="422"/>
+    <row r="423"/>
+    <row r="424"/>
+    <row r="425"/>
+    <row r="426"/>
+    <row r="427"/>
+    <row r="428"/>
+    <row r="429"/>
+    <row r="430"/>
+    <row r="431"/>
+    <row r="432"/>
+    <row r="433"/>
+    <row r="434"/>
+    <row r="435"/>
+    <row r="436"/>
+    <row r="437"/>
+    <row r="438"/>
+    <row r="439"/>
+    <row r="440"/>
+    <row r="441"/>
+    <row r="442"/>
+    <row r="443"/>
+    <row r="444"/>
+    <row r="445"/>
+    <row r="446"/>
+    <row r="447"/>
+    <row r="448"/>
+    <row r="449"/>
+    <row r="450"/>
+    <row r="451"/>
+    <row r="452"/>
+    <row r="453"/>
+    <row r="454"/>
+    <row r="455"/>
+    <row r="456"/>
+    <row r="457"/>
+    <row r="458"/>
+    <row r="459"/>
+    <row r="460"/>
+    <row r="461"/>
+    <row r="462"/>
+    <row r="463"/>
+    <row r="464"/>
+    <row r="465"/>
+    <row r="466"/>
+    <row r="467"/>
+    <row r="468"/>
+    <row r="469"/>
+    <row r="470"/>
+    <row r="471"/>
+    <row r="472"/>
+    <row r="473"/>
+    <row r="474"/>
+    <row r="475"/>
+    <row r="476"/>
+    <row r="477"/>
+    <row r="478"/>
+    <row r="479"/>
+    <row r="480"/>
+    <row r="481"/>
+    <row r="482"/>
+    <row r="483"/>
+    <row r="484"/>
+    <row r="485"/>
+    <row r="486"/>
+    <row r="487"/>
+    <row r="488"/>
+    <row r="489"/>
+    <row r="490"/>
+    <row r="491"/>
+    <row r="492"/>
+    <row r="493"/>
+    <row r="494"/>
+    <row r="495"/>
+    <row r="496"/>
+    <row r="497"/>
+    <row r="498"/>
+    <row r="499"/>
+    <row r="500"/>
+    <row r="501"/>
+    <row r="502"/>
+    <row r="503"/>
+    <row r="504"/>
+    <row r="505"/>
+    <row r="506"/>
+    <row r="507"/>
+    <row r="508"/>
+    <row r="509"/>
+    <row r="510"/>
+    <row r="511"/>
+    <row r="512"/>
+    <row r="513"/>
+    <row r="514"/>
+    <row r="515"/>
+    <row r="516"/>
+    <row r="517"/>
+    <row r="518"/>
+    <row r="519"/>
+    <row r="520"/>
+    <row r="521"/>
+    <row r="522"/>
+    <row r="523"/>
+    <row r="524"/>
+    <row r="525"/>
+    <row r="526"/>
+    <row r="527"/>
+    <row r="528"/>
+    <row r="529"/>
+    <row r="530"/>
+    <row r="531"/>
+    <row r="532"/>
+    <row r="533"/>
+    <row r="534"/>
+    <row r="535"/>
+    <row r="536"/>
+    <row r="537"/>
+    <row r="538"/>
+    <row r="539"/>
+    <row r="540"/>
+    <row r="541"/>
+    <row r="542"/>
+    <row r="543"/>
+    <row r="544"/>
+    <row r="545"/>
+    <row r="546"/>
+    <row r="547"/>
+    <row r="548"/>
+    <row r="549"/>
+    <row r="550"/>
+    <row r="551"/>
+    <row r="552"/>
+    <row r="553"/>
+    <row r="554"/>
+    <row r="555"/>
+    <row r="556"/>
+    <row r="557"/>
+    <row r="558"/>
+    <row r="559"/>
+    <row r="560"/>
+    <row r="561"/>
+    <row r="562"/>
+    <row r="563"/>
+    <row r="564"/>
+    <row r="565"/>
+    <row r="566"/>
+    <row r="567"/>
+    <row r="568"/>
+    <row r="569"/>
     <row r="570">
       <c r="J570" s="92" t="n"/>
     </row>
@@ -21110,7 +21544,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem (Back)</t>
+          <t>Proxy Delhaize Denderhoutem</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -21174,7 +21608,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>AD Aartselar (4 Back)</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -22710,7 +23144,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem (Back)</t>
+          <t>Proxy Delhaize Denderhoutem</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -23062,7 +23496,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>AD Aartselar (4 Back)</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -24182,7 +24616,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem (Back)</t>
+          <t>Proxy Delhaize Denderhoutem</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -25078,7 +25512,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>AD Aartselar (4 Back)</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -25526,7 +25960,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>AD Aartselar (1 Top)</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -25558,7 +25992,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem (Top)</t>
+          <t>Proxy Delhaize Denderhoutem</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -25942,7 +26376,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem (Back)</t>
+          <t>Proxy Delhaize Denderhoutem</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -26134,7 +26568,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem (Top)</t>
+          <t>Proxy Delhaize Denderhoutem</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -26198,7 +26632,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>AD Aartselar (4 Back)</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -27990,7 +28424,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem (Top)</t>
+          <t>Proxy Delhaize Denderhoutem</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -28022,7 +28456,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>AD Aartselar (1 Top)</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -28054,7 +28488,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>AD Aartselar (4 Back)</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -28598,7 +29032,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>AD Aartselar (4 Top)</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -28822,7 +29256,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem (Back)</t>
+          <t>Proxy Delhaize Denderhoutem</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -29206,7 +29640,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Spar Dadizele (2nd)</t>
+          <t>Spar Dadizele</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -29494,7 +29928,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem (Top)</t>
+          <t>Proxy Delhaize Denderhoutem</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -29526,7 +29960,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>AD Aartselar (1 Top)</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -29654,7 +30088,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>AD Aartselar (4 Back)</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -29814,7 +30248,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>PLUS Klazienaveen Fischer</t>
+          <t>Plus Klazienaveen Fischer</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -30710,7 +31144,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>PLUS Klazienaveen</t>
+          <t>Plus Klazienaveen Fischer</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -31286,7 +31720,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>spar Dadizele</t>
+          <t>Spar Dadizele</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -32630,7 +33064,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>AD Delhaize Aartselaar</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -32662,7 +33096,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>AD Delhaize Aartselaar</t>
+          <t>AD Aartselar</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -34058,7 +34492,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderleeuw</t>
+          <t>Proxy Delhaize Denderleew</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -36869,7 +37303,7 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>PLUS Simpelveld Schouteten</t>
+          <t>Plus Simpelveld Schouteten</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
@@ -36901,7 +37335,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>PLUS Simpelveld Schouteten</t>
+          <t>Plus Simpelveld Schouteten</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
@@ -41108,7 +41542,7 @@
       </c>
       <c r="B662" t="inlineStr">
         <is>
-          <t>PLUS Simpelveld Schouteten</t>
+          <t>Plus Simpelveld Schouteten</t>
         </is>
       </c>
       <c r="C662" t="inlineStr">

</xml_diff>

<commit_message>
Rename AD Delhaize X -> AD X and fix other project name variants
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -10496,7 +10496,7 @@
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Sint Lenaarts</t>
+          <t>AD Sint Lenaarts</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -10554,7 +10554,7 @@
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Fernelmont</t>
+          <t>AD Fernelmont</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -10728,7 +10728,7 @@
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve"> AD Delhaize Asse</t>
+          <t>AD Asse</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -10903,7 +10903,7 @@
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Hazegras</t>
+          <t>AD Hazegras</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -10960,7 +10960,7 @@
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve"> AD Delhaize Herselt</t>
+          <t>AD Herselt</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -11074,7 +11074,7 @@
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Sint Katelijne Waver</t>
+          <t>AD Sint Katelijne Waver</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -11139,7 +11139,7 @@
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Pallieter</t>
+          <t>AD Pallieter</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -11204,7 +11204,7 @@
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Itegem</t>
+          <t>AD Itegem</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -11269,7 +11269,7 @@
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Kluisbergen</t>
+          <t>AD Kluisbergen</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -11383,7 +11383,7 @@
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Wezemaal</t>
+          <t>AD Wezemaal</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -11513,7 +11513,7 @@
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Tielt-Winge</t>
+          <t>AD Tielt-Winge</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -11583,7 +11583,7 @@
     <row r="24">
       <c r="A24" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Dessel</t>
+          <t>AD Dessel</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -11648,7 +11648,7 @@
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="85" t="inlineStr">
         <is>
-          <t>AD Delhaize Kessel-Lo</t>
+          <t>AD Kessel-Lo</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -33000,7 +33000,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>AD Delhaize Nederename</t>
+          <t>AD Nederename</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -34524,7 +34524,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>AD Delhaize Denderleeuw</t>
+          <t>AD Denderleeuw</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
@@ -34556,7 +34556,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>AD Delhaize Retie</t>
+          <t>AD Retie</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -34588,7 +34588,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>AD Delhaize Arendonk</t>
+          <t>AD Arendonk</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -34652,7 +34652,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>AD Delhaize Watersport</t>
+          <t>AD Watersport</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
@@ -34684,7 +34684,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>AD Delhaize Bellegem</t>
+          <t>AD Bellegem</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -34716,7 +34716,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>AD Delhaize Kalmthout</t>
+          <t>AD Kalmthout</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
@@ -34748,7 +34748,7 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>AD Delhaize Grimbergen</t>
+          <t>AD Grimbergen</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
@@ -34780,7 +34780,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>AD Delhaize Halle</t>
+          <t>AD Halle</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -34876,7 +34876,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>AD Delhaize Deurne</t>
+          <t>AD Deurne</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
@@ -36028,7 +36028,7 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>AD Delhaize Geraardsbergen</t>
+          <t>AD Geraardsbergen</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
@@ -36092,7 +36092,7 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>AD Delhaize Zottegem</t>
+          <t>AD Zottegem</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
@@ -36570,7 +36570,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>AD Delhaize Borgerhout</t>
+          <t>AD Borgerhout</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
@@ -38004,7 +38004,7 @@
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>AD Delhaize Kessel-Lo</t>
+          <t>AD Kessel-Lo</t>
         </is>
       </c>
       <c r="C553" t="inlineStr">
@@ -38036,7 +38036,7 @@
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>AD Delhaize Dessel</t>
+          <t>AD Dessel</t>
         </is>
       </c>
       <c r="C554" t="inlineStr">
@@ -38068,7 +38068,7 @@
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>AD Delhaize Tielt-Winge</t>
+          <t>AD Tielt-Winge</t>
         </is>
       </c>
       <c r="C555" t="inlineStr">
@@ -38132,7 +38132,7 @@
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>AD Delhaize Wezemaal</t>
+          <t>AD Wezemaal</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
@@ -38196,7 +38196,7 @@
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>AD Delhaize Kluisbergen</t>
+          <t>AD Kluisbergen</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
@@ -38228,7 +38228,7 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>AD Delhaize Itegem</t>
+          <t>AD Itegem</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
@@ -38260,7 +38260,7 @@
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>AD Delhaize Pallieter</t>
+          <t>AD Pallieter</t>
         </is>
       </c>
       <c r="C561" t="inlineStr">
@@ -38292,7 +38292,7 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>AD Delhaize Sint Katelijne Waver</t>
+          <t>AD Sint Katelijne Waver</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
@@ -38324,7 +38324,7 @@
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t xml:space="preserve"> AD Delhaize Bloemmolens</t>
+          <t>AD Bloemmolens</t>
         </is>
       </c>
       <c r="C563" t="inlineStr">
@@ -38356,7 +38356,7 @@
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t xml:space="preserve"> AD Delhaize Herselt</t>
+          <t>AD Herselt</t>
         </is>
       </c>
       <c r="C564" t="inlineStr">
@@ -38388,7 +38388,7 @@
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>AD Delhaize Hazegras</t>
+          <t>AD Hazegras</t>
         </is>
       </c>
       <c r="C565" t="inlineStr">
@@ -40744,7 +40744,7 @@
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>AD Delhaize Sint Lenaarts</t>
+          <t>AD Sint Lenaarts</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
@@ -40776,7 +40776,7 @@
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>AD Delhaize Fernelmont</t>
+          <t>AD Fernelmont</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">

</xml_diff>

<commit_message>
Add Coop Bert Stuut and Jumbo Eindhoven Boschdijk renames; run standardization (35 cells renamed)
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -19480,7 +19480,7 @@
     <row r="133">
       <c r="A133" s="73" t="inlineStr">
         <is>
-          <t>JUMBO Eindhoven Boschdijk</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="B133" s="31" t="inlineStr">
@@ -21000,7 +21000,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Coop Bert Stuut (back)</t>
+          <t>Coop Bert Stuut</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -21864,7 +21864,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Jumbo Eindhoven Bosdijk</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -21896,7 +21896,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Coop bert stuut (Top)</t>
+          <t>Coop Bert Stuut</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -22472,7 +22472,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Coop Bert Stuut (back)</t>
+          <t>Coop Bert Stuut</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -23592,7 +23592,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Jumbo Eindhoven Bosdijk</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -23624,7 +23624,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Coop bert stuut (Top)</t>
+          <t>Coop Bert Stuut</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -23976,7 +23976,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Coop Bert Stuut (back)</t>
+          <t>Coop Bert Stuut</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -24520,7 +24520,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Jumbo Eindhoven Bosdijk (from side to TD)</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -25576,7 +25576,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Jumbo Eindhoven Bosdijk</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -25608,7 +25608,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Coop bert stuut (Top)</t>
+          <t>Coop Bert Stuut</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -27784,7 +27784,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Jumbo Eindhoven Bosdijk</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -30120,7 +30120,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Jumbo Eindhoven Bosdijk</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -30952,7 +30952,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Jumbo Eindhoven Bosdijk</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -37876,7 +37876,7 @@
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>JUMBO Eindhoven Boschdijk</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
@@ -40933,7 +40933,7 @@
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>Edeka Kusnezow-Lewandowski - Langerwehe</t>
+          <t>Edeka Kusnezow-Lewandowski Langerwehe</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
@@ -40962,7 +40962,7 @@
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Edeka Vogel-Lewandowski - Dueren</t>
+          <t>Edeka Vogel-Lewandowski Dueren</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
@@ -40991,7 +40991,7 @@
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>Edeka Vogel - Dueren</t>
+          <t>Edeka Vogel Dueren</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
@@ -41020,7 +41020,7 @@
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>Edeka Billstein - Wuppertal</t>
+          <t>Edeka Billstein Wuppertal</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
@@ -41049,7 +41049,7 @@
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Edeka Hoevener - Langenfeld</t>
+          <t>Edeka Hoevener Langenfeld</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
@@ -41078,7 +41078,7 @@
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Edeka Paschmann - Muelheim</t>
+          <t>Edeka Paschmann Muelheim</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
@@ -41107,7 +41107,7 @@
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Edeka Steren - Sulingen</t>
+          <t>Edeka Steren Sulingen</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
@@ -41136,7 +41136,7 @@
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Edeka Rath - Grevenbroich</t>
+          <t>Edeka Rath Grevenbroich</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
@@ -41571,7 +41571,7 @@
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>JUMBO Eindhoven Boschdijk</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">

</xml_diff>

<commit_message>
Add bulk project name standardizations (Proxy Delhaize→Proxy, case fixes, typos) — 254 cells total
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -10318,7 +10318,7 @@
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="85" t="inlineStr">
         <is>
-          <t>EDEKA DORTMUND</t>
+          <t>Edeka Dortmund</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -10612,7 +10612,7 @@
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Proxy Delhaize OOIGEM</t>
+          <t>Proxy Ooigem</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -11326,7 +11326,7 @@
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Proxy Delhaize Veltem</t>
+          <t>Proxy Veltem</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -11448,7 +11448,7 @@
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="181" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Durme (Heads)</t>
+          <t>Proxy Durme (Heads)</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -13246,7 +13246,7 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>CM Waregram</t>
+          <t>CM Waregem</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -13318,7 +13318,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Sint-Amandsberg</t>
+          <t>Proxy Sint-Amandsberg</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -13608,7 +13608,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Sint-Lievens-Houtem</t>
+          <t>Proxy Sint-Lievens-Houtem</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -13752,7 +13752,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Westkerke</t>
+          <t>Proxy Westkerke</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
@@ -14040,7 +14040,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Veerle</t>
+          <t>Proxy Veerle</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -14112,7 +14112,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Westerlo</t>
+          <t>Proxy Westerlo</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -14400,7 +14400,7 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>AD ARENDONK</t>
+          <t>AD Arendonk</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -14544,7 +14544,7 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>AD Denderleew</t>
+          <t>AD Denderleeuw</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -14616,7 +14616,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderleew</t>
+          <t>Proxy Denderleew</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
@@ -15050,7 +15050,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Langemark</t>
+          <t>Proxy Langemark</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -15462,7 +15462,7 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Beerzel</t>
+          <t>Proxy Beerzel</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -15529,7 +15529,7 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Sint Jan in Eremo</t>
+          <t>Proxy Sint Jan in Eremo</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -15876,7 +15876,7 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Fléron</t>
+          <t>Proxy Fléron</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
@@ -17472,7 +17472,7 @@
     <row r="107">
       <c r="A107" s="17" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Leest</t>
+          <t>Proxy Leest</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -17545,7 +17545,7 @@
     <row r="108">
       <c r="A108" s="17" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Meeuwen</t>
+          <t>Proxy Meeuwen</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
@@ -18468,7 +18468,7 @@
     <row r="120">
       <c r="A120" s="73" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Berchem</t>
+          <t>Proxy Berchem</t>
         </is>
       </c>
       <c r="B120" s="31" t="inlineStr">
@@ -18624,7 +18624,7 @@
     <row r="122">
       <c r="A122" s="17" t="inlineStr">
         <is>
-          <t>Spar Denderleew (vim3)</t>
+          <t>Spar Denderleew</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
@@ -18701,7 +18701,7 @@
     <row r="123">
       <c r="A123" s="19" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
@@ -19029,7 +19029,7 @@
     <row r="127">
       <c r="A127" s="17" t="inlineStr">
         <is>
-          <t>CM Alma mol</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="B127" s="7" t="inlineStr">
@@ -19351,7 +19351,7 @@
     <row r="131">
       <c r="A131" s="73" t="inlineStr">
         <is>
-          <t>JUMBO 's Gravendeel van der Hoek</t>
+          <t>Jumbo Gravendeel Van Der Hoek</t>
         </is>
       </c>
       <c r="B131" s="31" t="inlineStr">
@@ -21128,7 +21128,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Muizen</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -21544,7 +21544,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -21928,7 +21928,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Coop Cockengen</t>
+          <t>Coop Kockengen</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -22152,7 +22152,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Plus kamerik Romijn</t>
+          <t>Plus Kamerik Romijn</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -22600,7 +22600,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Muizen</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -22792,7 +22792,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CM Alma mol</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -22856,7 +22856,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Jumbo Groningen pestman</t>
+          <t>Jumbo Groningen Pestman</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -22920,7 +22920,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Jumbo Gravendeel</t>
+          <t>Jumbo Gravendeel Van Der Hoek</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -23144,7 +23144,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -24072,7 +24072,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Muizen</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -24328,7 +24328,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Plus kamerik Romijn</t>
+          <t>Plus Kamerik Romijn</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -24616,7 +24616,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -24872,7 +24872,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>CM Alma mol</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -24904,7 +24904,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Jumbo Groningen pestman</t>
+          <t>Jumbo Groningen Pestman</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -24968,7 +24968,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Jumbo Gravendeel</t>
+          <t>Jumbo Gravendeel Van Der Hoek</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -25992,7 +25992,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -26024,7 +26024,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Berchem</t>
+          <t>Proxy Berchem</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -26120,7 +26120,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Muizen</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -26344,7 +26344,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CM Alma mol</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -26376,7 +26376,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -26472,7 +26472,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Alvo Konitch</t>
+          <t>Alvo Kontich</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -26568,7 +26568,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -26856,7 +26856,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Muizen</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -27528,7 +27528,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Plus Simpleveld Schouteden</t>
+          <t>Plus Simpelveld Schouteten</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -27720,7 +27720,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>CM Alma mol</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -28072,7 +28072,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Plus Simpelveld Schouteden</t>
+          <t>Plus Simpelveld Schouteten</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -28392,7 +28392,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Berchem</t>
+          <t>Proxy Berchem</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -28424,7 +28424,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -28616,7 +28616,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Meeuwen</t>
+          <t>Proxy Meeuwen</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -28744,7 +28744,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Plus kamerik Romijn</t>
+          <t>Plus Kamerik Romijn</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -29256,7 +29256,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -29512,7 +29512,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Leest</t>
+          <t>Proxy Leest</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -29544,7 +29544,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Grootzand</t>
+          <t>Proxy Grootzand</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -29768,7 +29768,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Muizen</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -29896,7 +29896,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Berchem</t>
+          <t>Proxy Berchem</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -29928,7 +29928,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -30056,7 +30056,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>CM Alma mol</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -30792,7 +30792,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Jumbo Gravendeel</t>
+          <t>Jumbo Gravendeel Van Der Hoek</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -30888,7 +30888,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Meeuwen</t>
+          <t>Proxy Meeuwen</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -31240,7 +31240,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>CM Alma mol</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -31464,7 +31464,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>JUMBO Olm Krimpen aan den Ijssel</t>
+          <t>Jumbo Olm Krimpen aan den Ijssel</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -31496,7 +31496,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>PLUS Landgraaf Arts</t>
+          <t>Plus Landgraaf Arts</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -31592,7 +31592,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Grootzand</t>
+          <t>Proxy Grootzand</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -31624,7 +31624,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Leest</t>
+          <t>Proxy Leest</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -31752,7 +31752,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Muizen</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -31880,7 +31880,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Berchem</t>
+          <t>Proxy Berchem</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -31912,7 +31912,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -32200,7 +32200,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>AH Dendemonde</t>
+          <t>AH Dendermonde</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -32232,7 +32232,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>AD Soumagune</t>
+          <t>AD Soumagne</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -32264,7 +32264,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Fléron</t>
+          <t>Proxy Fléron</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -32776,7 +32776,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Meeuwen</t>
+          <t>Proxy Meeuwen</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -32968,7 +32968,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Sint Jan in Eremo</t>
+          <t>Proxy Sint Jan in Eremo</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
@@ -33224,7 +33224,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>CM Alma mol</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -33378,7 +33378,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Beerzel</t>
+          <t>Proxy Beerzel</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -33724,7 +33724,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Grootzand</t>
+          <t>Proxy Grootzand</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
@@ -33756,7 +33756,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Leest</t>
+          <t>Proxy Leest</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -33884,7 +33884,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Muizen</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -33980,7 +33980,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -34044,7 +34044,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Staden</t>
+          <t>Proxy Staden</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -34076,7 +34076,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Langemark</t>
+          <t>Proxy Langemark</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -34108,7 +34108,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>AH Dendemonde</t>
+          <t>AH Dendermonde</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -34492,7 +34492,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderleew</t>
+          <t>Proxy Denderleew</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -34812,7 +34812,7 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Westerlo</t>
+          <t>Proxy Westerlo</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
@@ -34844,7 +34844,7 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Veerle</t>
+          <t>Proxy Veerle</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
@@ -34940,7 +34940,7 @@
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Fléron</t>
+          <t>Proxy Fléron</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
@@ -35132,7 +35132,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Westkerke</t>
+          <t>Proxy Westkerke</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
@@ -35164,7 +35164,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>AD SOUMAGANE</t>
+          <t>AD Soumagne</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
@@ -35452,7 +35452,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Sint-Amandsberg</t>
+          <t>Proxy Sint-Amandsberg</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
@@ -35740,7 +35740,7 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Sint Jan in Eremo</t>
+          <t>Proxy Sint Jan in Eremo</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
@@ -35964,7 +35964,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>CM Alma mol</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
@@ -36234,7 +36234,7 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>PLUS Landgraaf Arts</t>
+          <t>Plus Landgraaf Arts</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
@@ -36596,7 +36596,7 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Staden</t>
+          <t>Proxy Staden</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
@@ -36628,7 +36628,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Langemark</t>
+          <t>Proxy Langemark</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
@@ -36724,7 +36724,7 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Beerzel</t>
+          <t>Proxy Beerzel</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
@@ -36948,7 +36948,7 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Grootzand</t>
+          <t>Proxy Grootzand</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
@@ -36980,7 +36980,7 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Leest</t>
+          <t>Proxy Leest</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
@@ -37102,7 +37102,7 @@
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Muizen</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
@@ -37195,7 +37195,7 @@
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
@@ -37524,7 +37524,7 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>AH Dendemonde</t>
+          <t>AH Dendermonde</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
@@ -38100,7 +38100,7 @@
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Durme</t>
+          <t>Proxy Durme</t>
         </is>
       </c>
       <c r="C556" t="inlineStr">
@@ -38164,7 +38164,7 @@
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Proxy Delhaize Veltem</t>
+          <t>Proxy Veltem</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
@@ -38420,7 +38420,7 @@
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Delhaize Belval LUXemburg</t>
+          <t>Delhaize Belval Luxemburg</t>
         </is>
       </c>
       <c r="C566" t="inlineStr">
@@ -38522,7 +38522,7 @@
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Sint Jan in Eremo</t>
+          <t>Proxy Sint Jan in Eremo</t>
         </is>
       </c>
       <c r="C569" t="inlineStr">
@@ -38802,7 +38802,7 @@
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>CM Waregram</t>
+          <t>CM Waregem</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
@@ -38837,7 +38837,7 @@
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Sint-Amandsberg</t>
+          <t>Proxy Sint-Amandsberg</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
@@ -38977,7 +38977,7 @@
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Sint-Lievens-Houtem</t>
+          <t>Proxy Sint-Lievens-Houtem</t>
         </is>
       </c>
       <c r="C582" t="inlineStr">
@@ -39222,7 +39222,7 @@
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Westkerke</t>
+          <t>Proxy Westkerke</t>
         </is>
       </c>
       <c r="C589" t="inlineStr">
@@ -39257,7 +39257,7 @@
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Westerlo</t>
+          <t>Proxy Westerlo</t>
         </is>
       </c>
       <c r="C590" t="inlineStr">
@@ -39327,7 +39327,7 @@
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>Spar Denderleew (vim3)</t>
+          <t>Spar Denderleew</t>
         </is>
       </c>
       <c r="D592" t="n">
@@ -39421,7 +39421,7 @@
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Veerle</t>
+          <t>Proxy Veerle</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
@@ -39561,7 +39561,7 @@
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>AD ARENDONK</t>
+          <t>AD Arendonk</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
@@ -39666,7 +39666,7 @@
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Fléron</t>
+          <t>Proxy Fléron</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
@@ -39771,7 +39771,7 @@
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Meeuwen</t>
+          <t>Proxy Meeuwen</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
@@ -39841,7 +39841,7 @@
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>JUMBO 's Gravendeel van der Hoek</t>
+          <t>Jumbo Gravendeel Van Der Hoek</t>
         </is>
       </c>
       <c r="C607" t="inlineStr">
@@ -39876,7 +39876,7 @@
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>AD Denderleew</t>
+          <t>AD Denderleeuw</t>
         </is>
       </c>
       <c r="C608" t="inlineStr">
@@ -39911,7 +39911,7 @@
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderleew</t>
+          <t>Proxy Denderleew</t>
         </is>
       </c>
       <c r="C609" t="inlineStr">
@@ -40051,7 +40051,7 @@
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>AH Merksem MAATJES_x000D_</t>
+          <t>AH Merksem MAATJES</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
@@ -40121,7 +40121,7 @@
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>AD Geraardsbergen_x000D_</t>
+          <t>AD Geraardsbergen</t>
         </is>
       </c>
       <c r="C615" t="inlineStr">
@@ -40191,7 +40191,7 @@
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>CM Alma mol</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="C617" t="inlineStr">
@@ -40552,7 +40552,7 @@
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Muizen</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
@@ -40584,7 +40584,7 @@
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>Proxy Delhaize Denderhoutem</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C630" t="inlineStr">
@@ -40616,7 +40616,7 @@
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proxy Delhaize Grootzand </t>
+          <t>Proxy Grootzand</t>
         </is>
       </c>
       <c r="C631" t="inlineStr">
@@ -40808,7 +40808,7 @@
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Proxy Delhaize OOIGEM</t>
+          <t>Proxy Ooigem</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
@@ -40840,7 +40840,7 @@
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Proxy Delhaize Wakken</t>
+          <t>Proxy Wakken</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
@@ -40991,7 +40991,7 @@
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>Edeka Vogel Dueren</t>
+          <t>Edeka Vogel-Lewandowski Dueren</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
@@ -41658,7 +41658,7 @@
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>EDEKA DORTMUND</t>
+          <t>Edeka Dortmund</t>
         </is>
       </c>
       <c r="C666" t="inlineStr">

</xml_diff>

<commit_message>
Merge variant project names (Plus Delft, Meerkerk, Maastricht Caberg, Jumbo Uden, Alma Geel, Eurospar, etc.)
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -16442,7 +16442,7 @@
     <row r="93">
       <c r="A93" s="14" t="inlineStr">
         <is>
-          <t>Alma Geel</t>
+          <t>CM Alma Geel</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
@@ -21416,7 +21416,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Plus Meerkerk (Back)</t>
+          <t>Plus Meerkerk</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -21800,7 +21800,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Plus Delft (4 Back)</t>
+          <t>Plus Delft</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -23016,7 +23016,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Plus Meerkerk (Back)</t>
+          <t>Plus Meerkerk</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -23432,7 +23432,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Plus Delft (1 Top)</t>
+          <t>Plus Delft</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -23528,7 +23528,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Plus Delft (4 Back)</t>
+          <t>Plus Delft</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -23752,7 +23752,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Jumbo Uden De Laak (Back)</t>
+          <t>Jumbo Uden De Laak</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -24104,7 +24104,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Plus Meerkerk (Top)</t>
+          <t>Plus Meerkerk</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -24232,7 +24232,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EuroSpar Denderleew</t>
+          <t>Eurospar Denderleew</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -24264,7 +24264,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Jumbo Uden De Laak (from Back to TD)</t>
+          <t>Jumbo Uden De Laak</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -24488,7 +24488,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Plus Maastricht Caberg  (from Back to TD)</t>
+          <t>Plus Maastricht Caberg</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -24680,7 +24680,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Plus Meerkerk (Back)</t>
+          <t>Plus Meerkerk</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -25256,7 +25256,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Jumbo Uden De Laak (Back)</t>
+          <t>Jumbo Uden De Laak</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -25288,7 +25288,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Plus Delft (1 Top)</t>
+          <t>Plus Delft</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -25544,7 +25544,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Plus Delft (4 Back)</t>
+          <t>Plus Delft</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -26280,7 +26280,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>EuroSpar Denderleew</t>
+          <t>Eurospar Denderleew</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -26824,7 +26824,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>EuroSpar Denderleew</t>
+          <t>Eurospar Denderleew</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -27080,7 +27080,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Jumbo Uden De Laak (Back)</t>
+          <t>Jumbo Uden De Laak</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -27656,7 +27656,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Plus langraaf Aarts extra checkouts</t>
+          <t>Plus Landgraaf Arts</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -28200,7 +28200,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Eurospar Dadizele (2nd)</t>
+          <t>Eurospar Dadizele</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -29992,7 +29992,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Jumbo Uden De Laak (Back)</t>
+          <t>Jumbo Uden De Laak</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -30024,7 +30024,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Jumbo Uden De Laak (Back)</t>
+          <t>Jumbo Uden De Laak</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -32648,7 +32648,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>Alma Geel</t>
+          <t>CM Alma Geel</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -32840,7 +32840,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>EuroSpar Denderleew</t>
+          <t>Eurospar Denderleew</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -35004,7 +35004,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>Alma Geel</t>
+          <t>CM Alma Geel</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
@@ -35292,7 +35292,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>Delhaize Sint-Lievens-Houtem</t>
+          <t>Proxy Sint-Lievens-Houtem</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
@@ -39736,7 +39736,7 @@
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>Alma Geel</t>
+          <t>CM Alma Geel</t>
         </is>
       </c>
       <c r="C604" t="inlineStr">

</xml_diff>

<commit_message>
Delete invoice #8667 rows and #8687 (cleanup); next invoice = 8674
</commit_message>
<xml_diff>
--- a/data/CaddyCheckProjectsInfo.xlsx
+++ b/data/CaddyCheckProjectsInfo.xlsx
@@ -19541,446 +19541,12 @@
         <v>46388</v>
       </c>
     </row>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
     <row r="180">
       <c r="J180" s="92" t="n"/>
     </row>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
     <row r="184">
       <c r="J184" s="78" t="n"/>
     </row>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
-    <row r="202"/>
-    <row r="203"/>
-    <row r="204"/>
-    <row r="205"/>
-    <row r="206"/>
-    <row r="207"/>
-    <row r="208"/>
-    <row r="209"/>
-    <row r="210"/>
-    <row r="211"/>
-    <row r="212"/>
-    <row r="213"/>
-    <row r="214"/>
-    <row r="215"/>
-    <row r="216"/>
-    <row r="217"/>
-    <row r="218"/>
-    <row r="219"/>
-    <row r="220"/>
-    <row r="221"/>
-    <row r="222"/>
-    <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
-    <row r="261"/>
-    <row r="262"/>
-    <row r="263"/>
-    <row r="264"/>
-    <row r="265"/>
-    <row r="266"/>
-    <row r="267"/>
-    <row r="268"/>
-    <row r="269"/>
-    <row r="270"/>
-    <row r="271"/>
-    <row r="272"/>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275"/>
-    <row r="276"/>
-    <row r="277"/>
-    <row r="278"/>
-    <row r="279"/>
-    <row r="280"/>
-    <row r="281"/>
-    <row r="282"/>
-    <row r="283"/>
-    <row r="284"/>
-    <row r="285"/>
-    <row r="286"/>
-    <row r="287"/>
-    <row r="288"/>
-    <row r="289"/>
-    <row r="290"/>
-    <row r="291"/>
-    <row r="292"/>
-    <row r="293"/>
-    <row r="294"/>
-    <row r="295"/>
-    <row r="296"/>
-    <row r="297"/>
-    <row r="298"/>
-    <row r="299"/>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302"/>
-    <row r="303"/>
-    <row r="304"/>
-    <row r="305"/>
-    <row r="306"/>
-    <row r="307"/>
-    <row r="308"/>
-    <row r="309"/>
-    <row r="310"/>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313"/>
-    <row r="314"/>
-    <row r="315"/>
-    <row r="316"/>
-    <row r="317"/>
-    <row r="318"/>
-    <row r="319"/>
-    <row r="320"/>
-    <row r="321"/>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324"/>
-    <row r="325"/>
-    <row r="326"/>
-    <row r="327"/>
-    <row r="328"/>
-    <row r="329"/>
-    <row r="330"/>
-    <row r="331"/>
-    <row r="332"/>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335"/>
-    <row r="336"/>
-    <row r="337"/>
-    <row r="338"/>
-    <row r="339"/>
-    <row r="340"/>
-    <row r="341"/>
-    <row r="342"/>
-    <row r="343"/>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
-    <row r="347"/>
-    <row r="348"/>
-    <row r="349"/>
-    <row r="350"/>
-    <row r="351"/>
-    <row r="352"/>
-    <row r="353"/>
-    <row r="354"/>
-    <row r="355"/>
-    <row r="356"/>
-    <row r="357"/>
-    <row r="358"/>
-    <row r="359"/>
-    <row r="360"/>
-    <row r="361"/>
-    <row r="362"/>
-    <row r="363"/>
-    <row r="364"/>
-    <row r="365"/>
-    <row r="366"/>
-    <row r="367"/>
-    <row r="368"/>
-    <row r="369"/>
-    <row r="370"/>
-    <row r="371"/>
-    <row r="372"/>
-    <row r="373"/>
-    <row r="374"/>
-    <row r="375"/>
-    <row r="376"/>
-    <row r="377"/>
-    <row r="378"/>
-    <row r="379"/>
-    <row r="380"/>
-    <row r="381"/>
-    <row r="382"/>
-    <row r="383"/>
-    <row r="384"/>
-    <row r="385"/>
-    <row r="386"/>
-    <row r="387"/>
-    <row r="388"/>
-    <row r="389"/>
-    <row r="390"/>
-    <row r="391"/>
-    <row r="392"/>
-    <row r="393"/>
-    <row r="394"/>
-    <row r="395"/>
-    <row r="396"/>
-    <row r="397"/>
-    <row r="398"/>
-    <row r="399"/>
-    <row r="400"/>
-    <row r="401"/>
-    <row r="402"/>
-    <row r="403"/>
-    <row r="404"/>
-    <row r="405"/>
-    <row r="406"/>
-    <row r="407"/>
-    <row r="408"/>
-    <row r="409"/>
-    <row r="410"/>
-    <row r="411"/>
-    <row r="412"/>
-    <row r="413"/>
-    <row r="414"/>
-    <row r="415"/>
-    <row r="416"/>
-    <row r="417"/>
-    <row r="418"/>
-    <row r="419"/>
-    <row r="420"/>
-    <row r="421"/>
-    <row r="422"/>
-    <row r="423"/>
-    <row r="424"/>
-    <row r="425"/>
-    <row r="426"/>
-    <row r="427"/>
-    <row r="428"/>
-    <row r="429"/>
-    <row r="430"/>
-    <row r="431"/>
-    <row r="432"/>
-    <row r="433"/>
-    <row r="434"/>
-    <row r="435"/>
-    <row r="436"/>
-    <row r="437"/>
-    <row r="438"/>
-    <row r="439"/>
-    <row r="440"/>
-    <row r="441"/>
-    <row r="442"/>
-    <row r="443"/>
-    <row r="444"/>
-    <row r="445"/>
-    <row r="446"/>
-    <row r="447"/>
-    <row r="448"/>
-    <row r="449"/>
-    <row r="450"/>
-    <row r="451"/>
-    <row r="452"/>
-    <row r="453"/>
-    <row r="454"/>
-    <row r="455"/>
-    <row r="456"/>
-    <row r="457"/>
-    <row r="458"/>
-    <row r="459"/>
-    <row r="460"/>
-    <row r="461"/>
-    <row r="462"/>
-    <row r="463"/>
-    <row r="464"/>
-    <row r="465"/>
-    <row r="466"/>
-    <row r="467"/>
-    <row r="468"/>
-    <row r="469"/>
-    <row r="470"/>
-    <row r="471"/>
-    <row r="472"/>
-    <row r="473"/>
-    <row r="474"/>
-    <row r="475"/>
-    <row r="476"/>
-    <row r="477"/>
-    <row r="478"/>
-    <row r="479"/>
-    <row r="480"/>
-    <row r="481"/>
-    <row r="482"/>
-    <row r="483"/>
-    <row r="484"/>
-    <row r="485"/>
-    <row r="486"/>
-    <row r="487"/>
-    <row r="488"/>
-    <row r="489"/>
-    <row r="490"/>
-    <row r="491"/>
-    <row r="492"/>
-    <row r="493"/>
-    <row r="494"/>
-    <row r="495"/>
-    <row r="496"/>
-    <row r="497"/>
-    <row r="498"/>
-    <row r="499"/>
-    <row r="500"/>
-    <row r="501"/>
-    <row r="502"/>
-    <row r="503"/>
-    <row r="504"/>
-    <row r="505"/>
-    <row r="506"/>
-    <row r="507"/>
-    <row r="508"/>
-    <row r="509"/>
-    <row r="510"/>
-    <row r="511"/>
-    <row r="512"/>
-    <row r="513"/>
-    <row r="514"/>
-    <row r="515"/>
-    <row r="516"/>
-    <row r="517"/>
-    <row r="518"/>
-    <row r="519"/>
-    <row r="520"/>
-    <row r="521"/>
-    <row r="522"/>
-    <row r="523"/>
-    <row r="524"/>
-    <row r="525"/>
-    <row r="526"/>
-    <row r="527"/>
-    <row r="528"/>
-    <row r="529"/>
-    <row r="530"/>
-    <row r="531"/>
-    <row r="532"/>
-    <row r="533"/>
-    <row r="534"/>
-    <row r="535"/>
-    <row r="536"/>
-    <row r="537"/>
-    <row r="538"/>
-    <row r="539"/>
-    <row r="540"/>
-    <row r="541"/>
-    <row r="542"/>
-    <row r="543"/>
-    <row r="544"/>
-    <row r="545"/>
-    <row r="546"/>
-    <row r="547"/>
-    <row r="548"/>
-    <row r="549"/>
-    <row r="550"/>
-    <row r="551"/>
-    <row r="552"/>
-    <row r="553"/>
-    <row r="554"/>
-    <row r="555"/>
-    <row r="556"/>
-    <row r="557"/>
-    <row r="558"/>
-    <row r="559"/>
-    <row r="560"/>
-    <row r="561"/>
-    <row r="562"/>
-    <row r="563"/>
-    <row r="564"/>
-    <row r="565"/>
-    <row r="566"/>
-    <row r="567"/>
-    <row r="568"/>
-    <row r="569"/>
     <row r="570">
       <c r="J570" s="92" t="n"/>
     </row>
@@ -20428,7 +19994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I666"/>
+  <dimension ref="A1:I660"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.5703125" bestFit="1" customWidth="1" style="54" min="1" max="1"/>
@@ -39323,23 +38889,34 @@
     </row>
     <row r="592" hidden="1">
       <c r="A592" t="n">
-        <v>8687</v>
+        <v>8664</v>
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>Spar Denderleew</t>
+          <t>AD Kalmthout</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Y6</t>
         </is>
       </c>
       <c r="D592" t="n">
-        <v>912</v>
+        <v>2280</v>
       </c>
       <c r="E592" t="n">
-        <v>4</v>
+        <v>10</v>
+      </c>
+      <c r="F592" s="201" t="n">
+        <v>45874</v>
       </c>
       <c r="G592" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H592" t="n">
+        <v>2025</v>
       </c>
       <c r="I592" t="n">
         <v>228</v>
@@ -39351,7 +38928,7 @@
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>AD Kalmthout</t>
+          <t>AD Grimbergen</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -39360,10 +38937,10 @@
         </is>
       </c>
       <c r="D593" t="n">
-        <v>2280</v>
+        <v>2964</v>
       </c>
       <c r="E593" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F593" s="201" t="n">
         <v>45874</v>
@@ -39386,7 +38963,7 @@
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>AD Grimbergen</t>
+          <t>Proxy Veerle</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
@@ -39395,10 +38972,10 @@
         </is>
       </c>
       <c r="D594" t="n">
-        <v>2964</v>
+        <v>1824</v>
       </c>
       <c r="E594" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F594" s="201" t="n">
         <v>45874</v>
@@ -39421,7 +38998,7 @@
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>Proxy Veerle</t>
+          <t>AD Halle</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
@@ -39430,10 +39007,10 @@
         </is>
       </c>
       <c r="D595" t="n">
-        <v>1824</v>
+        <v>3192</v>
       </c>
       <c r="E595" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F595" s="201" t="n">
         <v>45874</v>
@@ -39456,7 +39033,7 @@
       </c>
       <c r="B596" t="inlineStr">
         <is>
-          <t>AD Halle</t>
+          <t>AD Bellegem</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
@@ -39465,10 +39042,10 @@
         </is>
       </c>
       <c r="D596" t="n">
-        <v>3192</v>
+        <v>1824</v>
       </c>
       <c r="E596" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F596" s="201" t="n">
         <v>45874</v>
@@ -39491,7 +39068,7 @@
       </c>
       <c r="B597" t="inlineStr">
         <is>
-          <t>AD Bellegem</t>
+          <t>AD Watersport</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
@@ -39500,10 +39077,10 @@
         </is>
       </c>
       <c r="D597" t="n">
-        <v>1824</v>
+        <v>3648</v>
       </c>
       <c r="E597" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F597" s="201" t="n">
         <v>45874</v>
@@ -39526,7 +39103,7 @@
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>AD Watersport</t>
+          <t>AD Arendonk</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
@@ -39535,10 +39112,10 @@
         </is>
       </c>
       <c r="D598" t="n">
-        <v>3648</v>
+        <v>2280</v>
       </c>
       <c r="E598" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F598" s="201" t="n">
         <v>45874</v>
@@ -39561,7 +39138,7 @@
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>AD Arendonk</t>
+          <t>AD Retie</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
@@ -39570,10 +39147,10 @@
         </is>
       </c>
       <c r="D599" t="n">
-        <v>2280</v>
+        <v>2736</v>
       </c>
       <c r="E599" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F599" s="201" t="n">
         <v>45874</v>
@@ -39596,7 +39173,7 @@
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>AD Retie</t>
+          <t>CM Square Marlow</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
@@ -39605,10 +39182,10 @@
         </is>
       </c>
       <c r="D600" t="n">
-        <v>2736</v>
+        <v>1368</v>
       </c>
       <c r="E600" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F600" s="201" t="n">
         <v>45874</v>
@@ -39631,7 +39208,7 @@
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>CM Square Marlow</t>
+          <t>Proxy Fléron</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
@@ -39640,10 +39217,10 @@
         </is>
       </c>
       <c r="D601" t="n">
-        <v>1368</v>
+        <v>2280</v>
       </c>
       <c r="E601" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F601" s="201" t="n">
         <v>45874</v>
@@ -39666,7 +39243,7 @@
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>Proxy Fléron</t>
+          <t>Cora Hornou</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
@@ -39675,10 +39252,10 @@
         </is>
       </c>
       <c r="D602" t="n">
-        <v>2280</v>
+        <v>2736</v>
       </c>
       <c r="E602" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F602" s="201" t="n">
         <v>45874</v>
@@ -39701,7 +39278,7 @@
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>Cora Hornou</t>
+          <t>CM Alma Geel</t>
         </is>
       </c>
       <c r="C603" t="inlineStr">
@@ -39710,10 +39287,10 @@
         </is>
       </c>
       <c r="D603" t="n">
-        <v>2736</v>
+        <v>1368</v>
       </c>
       <c r="E603" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F603" s="201" t="n">
         <v>45874</v>
@@ -39736,7 +39313,7 @@
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>CM Alma Geel</t>
+          <t>Proxy Meeuwen</t>
         </is>
       </c>
       <c r="C604" t="inlineStr">
@@ -39745,10 +39322,10 @@
         </is>
       </c>
       <c r="D604" t="n">
-        <v>1368</v>
+        <v>1824</v>
       </c>
       <c r="E604" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F604" s="201" t="n">
         <v>45874</v>
@@ -39771,7 +39348,7 @@
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>Proxy Meeuwen</t>
+          <t>CM Alma Lommel</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
@@ -39780,10 +39357,10 @@
         </is>
       </c>
       <c r="D605" t="n">
-        <v>1824</v>
+        <v>912</v>
       </c>
       <c r="E605" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F605" s="201" t="n">
         <v>45874</v>
@@ -39806,7 +39383,7 @@
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>CM Alma Lommel</t>
+          <t>Jumbo Gravendeel Van Der Hoek</t>
         </is>
       </c>
       <c r="C606" t="inlineStr">
@@ -39815,10 +39392,10 @@
         </is>
       </c>
       <c r="D606" t="n">
-        <v>912</v>
+        <v>684</v>
       </c>
       <c r="E606" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F606" s="201" t="n">
         <v>45874</v>
@@ -39841,7 +39418,7 @@
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>Jumbo Gravendeel Van Der Hoek</t>
+          <t>AD Denderleeuw</t>
         </is>
       </c>
       <c r="C607" t="inlineStr">
@@ -39850,10 +39427,10 @@
         </is>
       </c>
       <c r="D607" t="n">
-        <v>684</v>
+        <v>2736</v>
       </c>
       <c r="E607" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F607" s="201" t="n">
         <v>45874</v>
@@ -39876,7 +39453,7 @@
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>AD Denderleeuw</t>
+          <t>Proxy Denderleew</t>
         </is>
       </c>
       <c r="C608" t="inlineStr">
@@ -39885,10 +39462,10 @@
         </is>
       </c>
       <c r="D608" t="n">
-        <v>2736</v>
+        <v>1140</v>
       </c>
       <c r="E608" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F608" s="201" t="n">
         <v>45874</v>
@@ -39911,7 +39488,7 @@
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>Proxy Denderleew</t>
+          <t>Merim Supermarket</t>
         </is>
       </c>
       <c r="C609" t="inlineStr">
@@ -39920,10 +39497,10 @@
         </is>
       </c>
       <c r="D609" t="n">
-        <v>1140</v>
+        <v>2280</v>
       </c>
       <c r="E609" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F609" s="201" t="n">
         <v>45874</v>
@@ -39946,7 +39523,7 @@
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>Merim Supermarket</t>
+          <t>AH Roeselare</t>
         </is>
       </c>
       <c r="C610" t="inlineStr">
@@ -39955,10 +39532,10 @@
         </is>
       </c>
       <c r="D610" t="n">
-        <v>2280</v>
+        <v>684</v>
       </c>
       <c r="E610" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F610" s="201" t="n">
         <v>45874</v>
@@ -39977,26 +39554,26 @@
     </row>
     <row r="611" hidden="1">
       <c r="A611" t="n">
-        <v>8664</v>
+        <v>8665</v>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>AH Roeselare</t>
+          <t>AD Zottegem</t>
         </is>
       </c>
       <c r="C611" t="inlineStr">
         <is>
-          <t>Y6</t>
+          <t>Y9</t>
         </is>
       </c>
       <c r="D611" t="n">
-        <v>684</v>
+        <v>2736</v>
       </c>
       <c r="E611" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F611" s="201" t="n">
-        <v>45874</v>
+        <v>46044</v>
       </c>
       <c r="G611" t="inlineStr">
         <is>
@@ -40016,7 +39593,7 @@
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>AD Zottegem</t>
+          <t>AH Merksem MAATJES</t>
         </is>
       </c>
       <c r="C612" t="inlineStr">
@@ -40025,10 +39602,10 @@
         </is>
       </c>
       <c r="D612" t="n">
-        <v>2736</v>
+        <v>912</v>
       </c>
       <c r="E612" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F612" s="201" t="n">
         <v>46044</v>
@@ -40051,7 +39628,7 @@
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>AH Merksem MAATJES</t>
+          <t>CM Alma Bilzen</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
@@ -40086,7 +39663,7 @@
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>CM Alma Bilzen</t>
+          <t>AD Geraardsbergen</t>
         </is>
       </c>
       <c r="C614" t="inlineStr">
@@ -40095,10 +39672,10 @@
         </is>
       </c>
       <c r="D614" t="n">
-        <v>912</v>
+        <v>1140</v>
       </c>
       <c r="E614" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F614" s="201" t="n">
         <v>46044</v>
@@ -40121,7 +39698,7 @@
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>AD Geraardsbergen</t>
+          <t>AD Harelbeke</t>
         </is>
       </c>
       <c r="C615" t="inlineStr">
@@ -40130,10 +39707,10 @@
         </is>
       </c>
       <c r="D615" t="n">
-        <v>1140</v>
+        <v>3648</v>
       </c>
       <c r="E615" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="F615" s="201" t="n">
         <v>46044</v>
@@ -40156,7 +39733,7 @@
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>AD Harelbeke</t>
+          <t>CM Alma Mol</t>
         </is>
       </c>
       <c r="C616" t="inlineStr">
@@ -40165,10 +39742,10 @@
         </is>
       </c>
       <c r="D616" t="n">
-        <v>3648</v>
+        <v>1368</v>
       </c>
       <c r="E616" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="F616" s="201" t="n">
         <v>46044</v>
@@ -40187,26 +39764,26 @@
     </row>
     <row r="617" hidden="1">
       <c r="A617" t="n">
-        <v>8665</v>
+        <v>8666</v>
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>CM Alma Mol</t>
+          <t>AD Zwevegem</t>
         </is>
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>Y9</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="D617" t="n">
-        <v>1368</v>
+        <v>3192</v>
       </c>
       <c r="E617" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="F617" s="201" t="n">
-        <v>46044</v>
+        <v>46048</v>
       </c>
       <c r="G617" t="inlineStr">
         <is>
@@ -40226,7 +39803,7 @@
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>AD Zwevegem</t>
+          <t xml:space="preserve">AD Deinze </t>
         </is>
       </c>
       <c r="C618" t="inlineStr">
@@ -40235,10 +39812,10 @@
         </is>
       </c>
       <c r="D618" t="n">
-        <v>3192</v>
+        <v>5016</v>
       </c>
       <c r="E618" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F618" s="201" t="n">
         <v>46048</v>
@@ -40256,54 +39833,29 @@
       </c>
     </row>
     <row r="619" hidden="1">
-      <c r="A619" t="n">
-        <v>8666</v>
-      </c>
-      <c r="B619" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AD Deinze </t>
-        </is>
-      </c>
-      <c r="C619" t="inlineStr">
-        <is>
-          <t>Y2</t>
-        </is>
-      </c>
-      <c r="D619" t="n">
-        <v>5016</v>
-      </c>
-      <c r="E619" t="n">
-        <v>22</v>
-      </c>
-      <c r="F619" s="201" t="n">
-        <v>46048</v>
-      </c>
-      <c r="G619" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H619" t="n">
-        <v>2025</v>
-      </c>
       <c r="I619" t="n">
         <v>228</v>
       </c>
     </row>
     <row r="620" hidden="1">
       <c r="A620" t="n">
-        <v>8667</v>
+        <v>8668</v>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>AD Wondelgem</t>
+        </is>
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>Y4</t>
+          <t>Y5</t>
         </is>
       </c>
       <c r="D620" t="n">
-        <v>684</v>
+        <v>2736</v>
       </c>
       <c r="E620" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G620" t="inlineStr">
         <is>
@@ -40318,29 +39870,56 @@
       </c>
     </row>
     <row r="621" hidden="1">
+      <c r="A621" t="n">
+        <v>8668</v>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>CM Elouges</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="D621" t="n">
+        <v>912</v>
+      </c>
+      <c r="E621" t="n">
+        <v>4</v>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H621" t="n">
+        <v>2025</v>
+      </c>
       <c r="I621" t="n">
         <v>228</v>
       </c>
     </row>
     <row r="622" hidden="1">
       <c r="A622" t="n">
-        <v>8667</v>
+        <v>8668</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t xml:space="preserve">AD Heist </t>
+          <t>CM St-Gillis-Waas</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>Y4</t>
+          <t>Y5</t>
         </is>
       </c>
       <c r="D622" t="n">
-        <v>4104</v>
+        <v>1140</v>
       </c>
       <c r="E622" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G622" t="inlineStr">
         <is>
@@ -40356,23 +39935,23 @@
     </row>
     <row r="623" hidden="1">
       <c r="A623" t="n">
-        <v>8667</v>
+        <v>8668</v>
       </c>
       <c r="B623" t="inlineStr">
         <is>
-          <t>AD Waregem</t>
+          <t>Proxy Muizen</t>
         </is>
       </c>
       <c r="C623" t="inlineStr">
         <is>
-          <t>Y4</t>
+          <t>Y5</t>
         </is>
       </c>
       <c r="D623" t="n">
-        <v>4560</v>
+        <v>1824</v>
       </c>
       <c r="E623" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="G623" t="inlineStr">
         <is>
@@ -40388,23 +39967,23 @@
     </row>
     <row r="624" hidden="1">
       <c r="A624" t="n">
-        <v>8667</v>
+        <v>8668</v>
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>AH Oudenaarde</t>
+          <t>Proxy Denderhoutem</t>
         </is>
       </c>
       <c r="C624" t="inlineStr">
         <is>
-          <t>Y4</t>
+          <t>Y5</t>
         </is>
       </c>
       <c r="D624" t="n">
-        <v>684</v>
+        <v>912</v>
       </c>
       <c r="E624" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G624" t="inlineStr">
         <is>
@@ -40420,23 +39999,23 @@
     </row>
     <row r="625" hidden="1">
       <c r="A625" t="n">
-        <v>8667</v>
+        <v>8668</v>
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>AH Waregem</t>
+          <t>Proxy Grootzand</t>
         </is>
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>Y4</t>
+          <t>Y5</t>
         </is>
       </c>
       <c r="D625" t="n">
-        <v>684</v>
+        <v>2280</v>
       </c>
       <c r="E625" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G625" t="inlineStr">
         <is>
@@ -40456,7 +40035,7 @@
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>AD Wondelgem</t>
+          <t>AD Zwijnaarde</t>
         </is>
       </c>
       <c r="C626" t="inlineStr">
@@ -40465,10 +40044,10 @@
         </is>
       </c>
       <c r="D626" t="n">
-        <v>2736</v>
+        <v>1596</v>
       </c>
       <c r="E626" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G626" t="inlineStr">
         <is>
@@ -40488,7 +40067,7 @@
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>CM Elouges</t>
+          <t xml:space="preserve">AH Schilde </t>
         </is>
       </c>
       <c r="C627" t="inlineStr">
@@ -40520,7 +40099,7 @@
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>CM St-Gillis-Waas</t>
+          <t>CM Oedelem</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
@@ -40529,10 +40108,10 @@
         </is>
       </c>
       <c r="D628" t="n">
-        <v>1140</v>
+        <v>912</v>
       </c>
       <c r="E628" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G628" t="inlineStr">
         <is>
@@ -40548,20 +40127,20 @@
     </row>
     <row r="629" hidden="1">
       <c r="A629" t="n">
-        <v>8668</v>
+        <v>8670</v>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>Proxy Muizen</t>
+          <t>AD Sint Lenaarts</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>Y5</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D629" t="n">
-        <v>1824</v>
+        <v>6224</v>
       </c>
       <c r="E629" t="n">
         <v>8</v>
@@ -40575,28 +40154,28 @@
         <v>2025</v>
       </c>
       <c r="I629" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="630" hidden="1">
       <c r="A630" t="n">
-        <v>8668</v>
+        <v>8670</v>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>Proxy Denderhoutem</t>
+          <t>AD Fernelmont</t>
         </is>
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>Y5</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D630" t="n">
-        <v>912</v>
+        <v>6224</v>
       </c>
       <c r="E630" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G630" t="inlineStr">
         <is>
@@ -40607,28 +40186,28 @@
         <v>2025</v>
       </c>
       <c r="I630" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="631" hidden="1">
       <c r="A631" t="n">
-        <v>8668</v>
+        <v>8670</v>
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>Proxy Grootzand</t>
+          <t>Proxy Ooigem</t>
         </is>
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>Y5</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D631" t="n">
-        <v>2280</v>
+        <v>6224</v>
       </c>
       <c r="E631" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G631" t="inlineStr">
         <is>
@@ -40639,28 +40218,28 @@
         <v>2025</v>
       </c>
       <c r="I631" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="632" hidden="1">
       <c r="A632" t="n">
-        <v>8668</v>
+        <v>8670</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>AD Zwijnaarde</t>
+          <t>Proxy Wakken</t>
         </is>
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>Y5</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D632" t="n">
-        <v>1596</v>
+        <v>6224</v>
       </c>
       <c r="E632" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G632" t="inlineStr">
         <is>
@@ -40671,28 +40250,28 @@
         <v>2025</v>
       </c>
       <c r="I632" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="633" hidden="1">
       <c r="A633" t="n">
-        <v>8668</v>
+        <v>8670</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t xml:space="preserve">AH Schilde </t>
+          <t>intermarché Heusy</t>
         </is>
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>Y5</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D633" t="n">
-        <v>912</v>
+        <v>7780</v>
       </c>
       <c r="E633" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G633" t="inlineStr">
         <is>
@@ -40703,28 +40282,28 @@
         <v>2025</v>
       </c>
       <c r="I633" t="n">
-        <v>228</v>
+        <v>778</v>
       </c>
     </row>
     <row r="634">
       <c r="A634" t="n">
-        <v>8668</v>
+        <v>8669</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>CM Oedelem</t>
+          <t xml:space="preserve"> Rewe Schorn - Bergheim</t>
         </is>
       </c>
       <c r="C634" t="inlineStr">
         <is>
-          <t>Y5</t>
+          <t>Paid Trial-0.5Y</t>
         </is>
       </c>
       <c r="D634" t="n">
-        <v>912</v>
+        <v>389</v>
       </c>
       <c r="E634" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G634" t="inlineStr">
         <is>
@@ -40734,29 +40313,26 @@
       <c r="H634" t="n">
         <v>2025</v>
       </c>
-      <c r="I634" t="n">
-        <v>228</v>
-      </c>
     </row>
     <row r="635">
       <c r="A635" t="n">
-        <v>8670</v>
+        <v>8669</v>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>AD Sint Lenaarts</t>
+          <t>Edeka Kusnezow-Lewandowski Langerwehe</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>Paid Trial-0.5Y</t>
         </is>
       </c>
       <c r="D635" t="n">
-        <v>6224</v>
+        <v>389</v>
       </c>
       <c r="E635" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G635" t="inlineStr">
         <is>
@@ -40766,29 +40342,26 @@
       <c r="H635" t="n">
         <v>2025</v>
       </c>
-      <c r="I635" t="n">
-        <v>778</v>
-      </c>
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>8670</v>
+        <v>8669</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>AD Fernelmont</t>
+          <t>Edeka Vogel-Lewandowski Dueren</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>Paid Trial-0.5Y</t>
         </is>
       </c>
       <c r="D636" t="n">
-        <v>6224</v>
+        <v>389</v>
       </c>
       <c r="E636" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G636" t="inlineStr">
         <is>
@@ -40798,29 +40371,26 @@
       <c r="H636" t="n">
         <v>2025</v>
       </c>
-      <c r="I636" t="n">
-        <v>778</v>
-      </c>
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>8670</v>
+        <v>8669</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>Proxy Ooigem</t>
+          <t>Edeka Vogel-Lewandowski Dueren</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>Paid Trial-0.5Y</t>
         </is>
       </c>
       <c r="D637" t="n">
-        <v>6224</v>
+        <v>389</v>
       </c>
       <c r="E637" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G637" t="inlineStr">
         <is>
@@ -40830,29 +40400,26 @@
       <c r="H637" t="n">
         <v>2025</v>
       </c>
-      <c r="I637" t="n">
-        <v>778</v>
-      </c>
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>8670</v>
+        <v>8669</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>Proxy Wakken</t>
+          <t>Edeka Billstein Wuppertal</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>Paid Trial-0.5Y</t>
         </is>
       </c>
       <c r="D638" t="n">
-        <v>6224</v>
+        <v>389</v>
       </c>
       <c r="E638" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G638" t="inlineStr">
         <is>
@@ -40862,29 +40429,26 @@
       <c r="H638" t="n">
         <v>2025</v>
       </c>
-      <c r="I638" t="n">
-        <v>778</v>
-      </c>
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>8670</v>
+        <v>8669</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>intermarché Heusy</t>
+          <t>Edeka Hoevener Langenfeld</t>
         </is>
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>Y1</t>
+          <t>Paid Trial-0.5Y</t>
         </is>
       </c>
       <c r="D639" t="n">
-        <v>7780</v>
+        <v>389</v>
       </c>
       <c r="E639" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G639" t="inlineStr">
         <is>
@@ -40893,9 +40457,6 @@
       </c>
       <c r="H639" t="n">
         <v>2025</v>
-      </c>
-      <c r="I639" t="n">
-        <v>778</v>
       </c>
     </row>
     <row r="640">
@@ -40904,7 +40465,7 @@
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Rewe Schorn - Bergheim</t>
+          <t>Edeka Paschmann Muelheim</t>
         </is>
       </c>
       <c r="C640" t="inlineStr">
@@ -40933,7 +40494,7 @@
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>Edeka Kusnezow-Lewandowski Langerwehe</t>
+          <t>Edeka Steren Sulingen</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
@@ -40962,7 +40523,7 @@
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>Edeka Vogel-Lewandowski Dueren</t>
+          <t>Edeka Rath Grevenbroich</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
@@ -40987,23 +40548,23 @@
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>8669</v>
+        <v>8671</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>Edeka Vogel-Lewandowski Dueren</t>
+          <t>CM Meer</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
         <is>
-          <t>Paid Trial-0.5Y</t>
+          <t>Y7</t>
         </is>
       </c>
       <c r="D643" t="n">
-        <v>389</v>
+        <v>1368</v>
       </c>
       <c r="E643" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G643" t="inlineStr">
         <is>
@@ -41011,28 +40572,28 @@
         </is>
       </c>
       <c r="H643" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>8669</v>
+        <v>8671</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>Edeka Billstein Wuppertal</t>
+          <t>AH Ninove</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
         <is>
-          <t>Paid Trial-0.5Y</t>
+          <t>Y7</t>
         </is>
       </c>
       <c r="D644" t="n">
-        <v>389</v>
+        <v>912</v>
       </c>
       <c r="E644" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G644" t="inlineStr">
         <is>
@@ -41040,28 +40601,28 @@
         </is>
       </c>
       <c r="H644" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>8669</v>
+        <v>8671</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>Edeka Hoevener Langenfeld</t>
+          <t>AH Dendermonde</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
         <is>
-          <t>Paid Trial-0.5Y</t>
+          <t>Y7</t>
         </is>
       </c>
       <c r="D645" t="n">
-        <v>389</v>
+        <v>912</v>
       </c>
       <c r="E645" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G645" t="inlineStr">
         <is>
@@ -41069,28 +40630,28 @@
         </is>
       </c>
       <c r="H645" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>8669</v>
+        <v>8671</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>Edeka Paschmann Muelheim</t>
+          <t>AH Rumbeke</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>Paid Trial-0.5Y</t>
+          <t>Y7</t>
         </is>
       </c>
       <c r="D646" t="n">
-        <v>389</v>
+        <v>912</v>
       </c>
       <c r="E646" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G646" t="inlineStr">
         <is>
@@ -41098,28 +40659,28 @@
         </is>
       </c>
       <c r="H646" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>8669</v>
+        <v>8671</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>Edeka Steren Sulingen</t>
+          <t>CM Sint-Niklaas</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
         <is>
-          <t>Paid Trial-0.5Y</t>
+          <t>Y7</t>
         </is>
       </c>
       <c r="D647" t="n">
-        <v>389</v>
+        <v>1596</v>
       </c>
       <c r="E647" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G647" t="inlineStr">
         <is>
@@ -41127,28 +40688,28 @@
         </is>
       </c>
       <c r="H647" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>8669</v>
+        <v>8671</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>Edeka Rath Grevenbroich</t>
+          <t>CM Zeebrugge</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
         <is>
-          <t>Paid Trial-0.5Y</t>
+          <t>Y7</t>
         </is>
       </c>
       <c r="D648" t="n">
-        <v>389</v>
+        <v>684</v>
       </c>
       <c r="E648" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G648" t="inlineStr">
         <is>
@@ -41156,28 +40717,28 @@
         </is>
       </c>
       <c r="H648" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>8671</v>
+        <v>8672</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>CM Meer</t>
+          <t>CM Hoboken Zuid</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
         <is>
-          <t>Y7</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="D649" t="n">
-        <v>1368</v>
+        <v>2736</v>
       </c>
       <c r="E649" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G649" t="inlineStr">
         <is>
@@ -41190,23 +40751,23 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>8671</v>
+        <v>8672</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>AH Ninove</t>
+          <t>CM Hoboken Kiosk</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
         <is>
-          <t>Y7</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="D650" t="n">
-        <v>912</v>
+        <v>2280</v>
       </c>
       <c r="E650" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G650" t="inlineStr">
         <is>
@@ -41219,23 +40780,23 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>8671</v>
+        <v>8672</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>AH Dendermonde</t>
+          <t>AD Heist-op-den-Berg</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t>Y7</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="D651" t="n">
-        <v>912</v>
+        <v>2280</v>
       </c>
       <c r="E651" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G651" t="inlineStr">
         <is>
@@ -41248,23 +40809,23 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>8671</v>
+        <v>8672</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>AH Rumbeke</t>
+          <t>AD Brecht</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>Y7</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="D652" t="n">
-        <v>912</v>
+        <v>2736</v>
       </c>
       <c r="E652" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G652" t="inlineStr">
         <is>
@@ -41277,23 +40838,23 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>8671</v>
+        <v>8672</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>CM Sint-Niklaas</t>
+          <t>AD Merksplas</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>Y7</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="D653" t="n">
-        <v>1596</v>
+        <v>1824</v>
       </c>
       <c r="E653" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G653" t="inlineStr">
         <is>
@@ -41306,23 +40867,23 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>8671</v>
+        <v>8672</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>CM Zeebrugge</t>
+          <t>AD GrootBijgaarden</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>Y7</t>
+          <t>Y2</t>
         </is>
       </c>
       <c r="D654" t="n">
-        <v>684</v>
+        <v>4560</v>
       </c>
       <c r="E654" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="G654" t="inlineStr">
         <is>
@@ -41339,7 +40900,7 @@
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>CM Hoboken Zuid</t>
+          <t>AD Vichte</t>
         </is>
       </c>
       <c r="C655" t="inlineStr">
@@ -41348,10 +40909,10 @@
         </is>
       </c>
       <c r="D655" t="n">
-        <v>2736</v>
+        <v>1824</v>
       </c>
       <c r="E655" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G655" t="inlineStr">
         <is>
@@ -41368,7 +40929,7 @@
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>CM Hoboken Kiosk</t>
+          <t>Plus Simpelveld Schouteten</t>
         </is>
       </c>
       <c r="C656" t="inlineStr">
@@ -41377,10 +40938,10 @@
         </is>
       </c>
       <c r="D656" t="n">
-        <v>2280</v>
+        <v>1140</v>
       </c>
       <c r="E656" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G656" t="inlineStr">
         <is>
@@ -41397,7 +40958,7 @@
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>AD Heist-op-den-Berg</t>
+          <t>Jumbo Eindhoven Boschdijk</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
@@ -41406,10 +40967,10 @@
         </is>
       </c>
       <c r="D657" t="n">
-        <v>2280</v>
+        <v>684</v>
       </c>
       <c r="E657" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G657" t="inlineStr">
         <is>
@@ -41422,23 +40983,23 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>8672</v>
+        <v>8673</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>AD Brecht</t>
+          <t>AD Anderlecht</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
         <is>
-          <t>Y2</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D658" t="n">
-        <v>2736</v>
+        <v>4668</v>
       </c>
       <c r="E658" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G658" t="inlineStr">
         <is>
@@ -41451,23 +41012,23 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>8672</v>
+        <v>8673</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>AD Merksplas</t>
+          <t>AD Burenvile</t>
         </is>
       </c>
       <c r="C659" t="inlineStr">
         <is>
-          <t>Y2</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D659" t="n">
-        <v>1824</v>
+        <v>1556</v>
       </c>
       <c r="E659" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G659" t="inlineStr">
         <is>
@@ -41480,23 +41041,23 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>8672</v>
+        <v>8673</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>AD GrootBijgaarden</t>
+          <t>Edeka Dortmund</t>
         </is>
       </c>
       <c r="C660" t="inlineStr">
         <is>
-          <t>Y2</t>
+          <t>Y1</t>
         </is>
       </c>
       <c r="D660" t="n">
-        <v>4560</v>
+        <v>1556</v>
       </c>
       <c r="E660" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G660" t="inlineStr">
         <is>
@@ -41507,180 +41068,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="661" ht="101.25" customHeight="1">
-      <c r="A661" t="n">
-        <v>8672</v>
-      </c>
-      <c r="B661" t="inlineStr">
-        <is>
-          <t>AD Vichte</t>
-        </is>
-      </c>
-      <c r="C661" t="inlineStr">
-        <is>
-          <t>Y2</t>
-        </is>
-      </c>
-      <c r="D661" t="n">
-        <v>1824</v>
-      </c>
-      <c r="E661" t="n">
-        <v>8</v>
-      </c>
-      <c r="G661" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H661" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="662">
-      <c r="A662" t="n">
-        <v>8672</v>
-      </c>
-      <c r="B662" t="inlineStr">
-        <is>
-          <t>Plus Simpelveld Schouteten</t>
-        </is>
-      </c>
-      <c r="C662" t="inlineStr">
-        <is>
-          <t>Y2</t>
-        </is>
-      </c>
-      <c r="D662" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E662" t="n">
-        <v>5</v>
-      </c>
-      <c r="G662" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H662" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="663">
-      <c r="A663" t="n">
-        <v>8672</v>
-      </c>
-      <c r="B663" t="inlineStr">
-        <is>
-          <t>Jumbo Eindhoven Boschdijk</t>
-        </is>
-      </c>
-      <c r="C663" t="inlineStr">
-        <is>
-          <t>Y2</t>
-        </is>
-      </c>
-      <c r="D663" t="n">
-        <v>684</v>
-      </c>
-      <c r="E663" t="n">
-        <v>3</v>
-      </c>
-      <c r="G663" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H663" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="664">
-      <c r="A664" t="n">
-        <v>8673</v>
-      </c>
-      <c r="B664" t="inlineStr">
-        <is>
-          <t>AD Anderlecht</t>
-        </is>
-      </c>
-      <c r="C664" t="inlineStr">
-        <is>
-          <t>Y1</t>
-        </is>
-      </c>
-      <c r="D664" t="n">
-        <v>4668</v>
-      </c>
-      <c r="E664" t="n">
-        <v>6</v>
-      </c>
-      <c r="G664" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H664" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="665">
-      <c r="A665" t="n">
-        <v>8673</v>
-      </c>
-      <c r="B665" t="inlineStr">
-        <is>
-          <t>AD Burenvile</t>
-        </is>
-      </c>
-      <c r="C665" t="inlineStr">
-        <is>
-          <t>Y1</t>
-        </is>
-      </c>
-      <c r="D665" t="n">
-        <v>1556</v>
-      </c>
-      <c r="E665" t="n">
-        <v>2</v>
-      </c>
-      <c r="G665" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H665" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="666">
-      <c r="A666" t="n">
-        <v>8673</v>
-      </c>
-      <c r="B666" t="inlineStr">
-        <is>
-          <t>Edeka Dortmund</t>
-        </is>
-      </c>
-      <c r="C666" t="inlineStr">
-        <is>
-          <t>Y1</t>
-        </is>
-      </c>
-      <c r="D666" t="n">
-        <v>1556</v>
-      </c>
-      <c r="E666" t="n">
-        <v>2</v>
-      </c>
-      <c r="G666" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H666" t="n">
-        <v>2026</v>
-      </c>
-    </row>
+    <row r="661" ht="101.25" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:I670">
     <filterColumn colId="2" hiddenButton="0" showButton="1">

</xml_diff>